<commit_message>
Atualização automática via Power Automate
</commit_message>
<xml_diff>
--- a/planilhao.xlsx
+++ b/planilhao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tcdf.sharepoint.com/sites/SAED/Shared Documents/General/SAED/Controles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4793" documentId="13_ncr:1_{C887EC22-7CD1-4717-84BE-7303F42C5C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91AC18CE-5373-4274-8C86-DE9552FD1390}"/>
+  <xr:revisionPtr revIDLastSave="4885" documentId="13_ncr:1_{C887EC22-7CD1-4717-84BE-7303F42C5C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B68FE8E-29DA-429B-AF65-C9F46B050110}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ações InCompany" sheetId="3" r:id="rId1"/>
@@ -23,73 +23,73 @@
     <sheet name="Dashboard Maratonas" sheetId="27" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ações InCompany'!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ações InCompany'!$A$1:$A$748</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Ações InCompany'!$A$1:$T$676</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <customWorkbookViews>
+    <customWorkbookView name="Filtro 41" guid="{CA3FE984-959D-4FD1-AD51-F273057287D0}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 40" guid="{32D42168-6533-486B-BA4F-1FCBEE1D5E70}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 43" guid="{983434C3-FA2A-4410-B75A-EB842981FB7E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 42" guid="{66204134-7843-4E4D-9132-12589B1C9904}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 45" guid="{37A81383-EB82-4415-9CA7-3B544A1BA6DF}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 44" guid="{466B00F4-CD06-4459-9EAD-5E099599461D}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 47" guid="{B3051128-E594-4E84-A90F-3E0AA1920164}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 46" guid="{426752F7-EFAA-494A-8C44-3FE740F51102}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 49" guid="{888656D7-51D7-4D86-82B1-69398E74949E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 48" guid="{437C4520-960F-4EE8-BC29-5EAC5035FDE9}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 3" guid="{34EB6BDD-DB10-46C3-8070-38A1FF20F467}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 2" guid="{DC0F290D-0110-4230-A92A-0C9FF5FA3573}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 1" guid="{69BC16F3-55B0-4A0A-9007-3B0C4D012204}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 7" guid="{E936EEA7-993F-4552-BBDF-E1DB0091DFDE}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 6" guid="{6A040256-BBC3-4938-A5D6-D77105714F23}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 5" guid="{1C752AA4-ECD6-4155-AAB6-DB036719A0D6}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 4" guid="{091F3115-1E32-40D6-93A0-F16A7E814F96}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 30" guid="{2AB5F1EE-8485-44BA-A278-7AE3DE9CF145}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 32" guid="{265C295C-DFB6-4951-B01D-86C18934578C}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 31" guid="{678EC2BA-6745-461E-BAC1-D09F77FA1062}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 34" guid="{C7C27644-1A5D-4074-B300-764545BFC964}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 33" guid="{0C325FD1-5773-4650-8B0D-3332A38760DC}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 36" guid="{DA4468DA-23DF-4CE6-A7A1-D96801F812A5}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 35" guid="{BD49A265-64CA-4E25-B77B-BEA5B216E8B0}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 38" guid="{6F970FA6-35FA-43B5-8000-ED45D53ABBFB}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 37" guid="{AB062F27-A6C8-47F1-BE53-0FF9CA1DEF53}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 39" guid="{AA5A0339-5E84-4A56-8746-33FE6401E32F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 19" guid="{F8DFD977-D486-42A2-ADDC-71E97C40849F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 61" guid="{02C55D31-8E27-44A2-A753-221185C3D450}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 60" guid="{3A0B7064-EFB6-42D3-AA59-F49B2C2E28A3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 62" guid="{BF3829F5-7BD2-40A9-9D59-6FA51DE0B5DA}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 21" guid="{A3242535-E588-41A5-A488-2E120680CF6E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 20" guid="{70652B29-1ABA-485A-9A80-A46DCDFDCA82}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 23" guid="{A1C80D12-5F51-43D3-B26D-C4E8E80E8CF2}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 22" guid="{371F802A-A094-48E0-BF99-0747C34D37B9}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 25" guid="{743E0231-3395-43B3-ADCA-F3A128F1B83A}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 9" guid="{2AF3BD90-56F5-45E9-AAA2-03E540B72567}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 24" guid="{9A493B68-EB00-440B-8491-378C02F67A40}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 8" guid="{7F93445C-3064-44FB-ABC5-E30DCF77756E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 27" guid="{23C9FC25-18F4-47EF-A3B5-759DEC27F9E9}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 26" guid="{3B6786E1-C731-4815-9553-455D14481DD3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 29" guid="{B5CEFD59-C042-4547-AAFF-F62EC921EEC6}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 28" guid="{1AB13F6B-0D74-43EC-B774-8B52A94E0814}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 50" guid="{5480ECB2-55D1-41C0-8514-F0684F861D24}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 52" guid="{560766DC-06F5-422D-B190-641D8FE5A38D}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 51" guid="{0F15AC02-A38D-4E8A-8C4B-DD7F2868099F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 54" guid="{FB245C5C-9A8F-416D-A134-0975CF96E595}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 10" guid="{633FA869-BC39-409D-BF13-F2C3CBB9EA93}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 53" guid="{2BB93E5B-65F1-4C09-BB9E-66343F5B3E82}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 56" guid="{1105711C-AABE-4812-8827-ED6089DCF11E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 12" guid="{19CACD21-710C-4D14-9ACE-063162C7120B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 55" guid="{D2A89341-BB3B-405B-B324-3BE49BB6E042}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 11" guid="{0904EB7B-8DCA-4D50-AD8B-0A671CE637AF}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 58" guid="{DA1621F1-9CA5-43AE-9A42-AC9D36F85B7D}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 14" guid="{ED877901-4C49-488E-89E7-42CF1935CA6E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 13" guid="{DF0241CF-B7E5-4FA7-B0C8-FA54D26D77D7}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 57" guid="{6BA1C58C-C21F-47F7-B022-0FEA98904E5F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 16" guid="{9C7682D3-C31F-4FE6-8766-BC418D960F41}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 59" guid="{B2B68F91-0ADB-423D-BEF9-757DCA540FDD}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 15" guid="{DDC390A9-8BCC-4E1B-8EE8-FEFD20C963E8}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
+    <customWorkbookView name="Filtro 18" guid="{990EC2BE-89D2-41CF-8152-E21202B6F8D8}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
     <customWorkbookView name="Filtro 17" guid="{77C5030A-63E1-4109-A4D5-32A3FB7E122A}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 18" guid="{990EC2BE-89D2-41CF-8152-E21202B6F8D8}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 15" guid="{DDC390A9-8BCC-4E1B-8EE8-FEFD20C963E8}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 59" guid="{B2B68F91-0ADB-423D-BEF9-757DCA540FDD}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 16" guid="{9C7682D3-C31F-4FE6-8766-BC418D960F41}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 57" guid="{6BA1C58C-C21F-47F7-B022-0FEA98904E5F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 13" guid="{DF0241CF-B7E5-4FA7-B0C8-FA54D26D77D7}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 14" guid="{ED877901-4C49-488E-89E7-42CF1935CA6E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 58" guid="{DA1621F1-9CA5-43AE-9A42-AC9D36F85B7D}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 11" guid="{0904EB7B-8DCA-4D50-AD8B-0A671CE637AF}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 55" guid="{D2A89341-BB3B-405B-B324-3BE49BB6E042}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 12" guid="{19CACD21-710C-4D14-9ACE-063162C7120B}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 56" guid="{1105711C-AABE-4812-8827-ED6089DCF11E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 53" guid="{2BB93E5B-65F1-4C09-BB9E-66343F5B3E82}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 10" guid="{633FA869-BC39-409D-BF13-F2C3CBB9EA93}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 54" guid="{FB245C5C-9A8F-416D-A134-0975CF96E595}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 51" guid="{0F15AC02-A38D-4E8A-8C4B-DD7F2868099F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 52" guid="{560766DC-06F5-422D-B190-641D8FE5A38D}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 50" guid="{5480ECB2-55D1-41C0-8514-F0684F861D24}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 28" guid="{1AB13F6B-0D74-43EC-B774-8B52A94E0814}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 29" guid="{B5CEFD59-C042-4547-AAFF-F62EC921EEC6}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 26" guid="{3B6786E1-C731-4815-9553-455D14481DD3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 27" guid="{23C9FC25-18F4-47EF-A3B5-759DEC27F9E9}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 8" guid="{7F93445C-3064-44FB-ABC5-E30DCF77756E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 24" guid="{9A493B68-EB00-440B-8491-378C02F67A40}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 9" guid="{2AF3BD90-56F5-45E9-AAA2-03E540B72567}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 25" guid="{743E0231-3395-43B3-ADCA-F3A128F1B83A}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 22" guid="{371F802A-A094-48E0-BF99-0747C34D37B9}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 23" guid="{A1C80D12-5F51-43D3-B26D-C4E8E80E8CF2}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 20" guid="{70652B29-1ABA-485A-9A80-A46DCDFDCA82}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 21" guid="{A3242535-E588-41A5-A488-2E120680CF6E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 62" guid="{BF3829F5-7BD2-40A9-9D59-6FA51DE0B5DA}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 60" guid="{3A0B7064-EFB6-42D3-AA59-F49B2C2E28A3}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 61" guid="{02C55D31-8E27-44A2-A753-221185C3D450}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 19" guid="{F8DFD977-D486-42A2-ADDC-71E97C40849F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 39" guid="{AA5A0339-5E84-4A56-8746-33FE6401E32F}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 37" guid="{AB062F27-A6C8-47F1-BE53-0FF9CA1DEF53}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 38" guid="{6F970FA6-35FA-43B5-8000-ED45D53ABBFB}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 35" guid="{BD49A265-64CA-4E25-B77B-BEA5B216E8B0}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 36" guid="{DA4468DA-23DF-4CE6-A7A1-D96801F812A5}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 33" guid="{0C325FD1-5773-4650-8B0D-3332A38760DC}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 34" guid="{C7C27644-1A5D-4074-B300-764545BFC964}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 31" guid="{678EC2BA-6745-461E-BAC1-D09F77FA1062}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 32" guid="{265C295C-DFB6-4951-B01D-86C18934578C}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 30" guid="{2AB5F1EE-8485-44BA-A278-7AE3DE9CF145}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 4" guid="{091F3115-1E32-40D6-93A0-F16A7E814F96}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 5" guid="{1C752AA4-ECD6-4155-AAB6-DB036719A0D6}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 6" guid="{6A040256-BBC3-4938-A5D6-D77105714F23}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 7" guid="{E936EEA7-993F-4552-BBDF-E1DB0091DFDE}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 1" guid="{69BC16F3-55B0-4A0A-9007-3B0C4D012204}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 2" guid="{DC0F290D-0110-4230-A92A-0C9FF5FA3573}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 3" guid="{34EB6BDD-DB10-46C3-8070-38A1FF20F467}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 48" guid="{437C4520-960F-4EE8-BC29-5EAC5035FDE9}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 49" guid="{888656D7-51D7-4D86-82B1-69398E74949E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 46" guid="{426752F7-EFAA-494A-8C44-3FE740F51102}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 47" guid="{B3051128-E594-4E84-A90F-3E0AA1920164}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 44" guid="{466B00F4-CD06-4459-9EAD-5E099599461D}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 45" guid="{37A81383-EB82-4415-9CA7-3B544A1BA6DF}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 42" guid="{66204134-7843-4E4D-9132-12589B1C9904}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 43" guid="{983434C3-FA2A-4410-B75A-EB842981FB7E}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 40" guid="{32D42168-6533-486B-BA4F-1FCBEE1D5E70}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
-    <customWorkbookView name="Filtro 41" guid="{CA3FE984-959D-4FD1-AD51-F273057287D0}" maximized="1" windowWidth="0" windowHeight="0" activeSheetId="0"/>
   </customWorkbookViews>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -167,7 +167,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6494" uniqueCount="2944">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6527" uniqueCount="2956">
   <si>
     <t>ID</t>
   </si>
@@ -8413,28 +8413,37 @@
     <t>21 e 22/05/2026</t>
   </si>
   <si>
+    <t>Em andamento</t>
+  </si>
+  <si>
+    <t>4141/2026</t>
+  </si>
+  <si>
+    <t>Fiscalizações Baseadas em Risco</t>
+  </si>
+  <si>
+    <t>08 a 12/06/2026</t>
+  </si>
+  <si>
+    <t>Reinaldo Alencar; Rogério Ribeiro</t>
+  </si>
+  <si>
+    <t>3685/2026</t>
+  </si>
+  <si>
+    <t>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T2</t>
+  </si>
+  <si>
+    <t>09 a 11/06/2026</t>
+  </si>
+  <si>
     <t>A realizar</t>
   </si>
   <si>
-    <t>4141/2026</t>
-  </si>
-  <si>
-    <t>Fiscalizações Baseadas em Risco</t>
-  </si>
-  <si>
-    <t>08 a 12/06/2026</t>
-  </si>
-  <si>
-    <t>Reinaldo Alencar; Rogério Ribeiro</t>
-  </si>
-  <si>
-    <t>3685/2026</t>
-  </si>
-  <si>
-    <t>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T2</t>
-  </si>
-  <si>
-    <t>09 a 11/06/2026</t>
+    <t>Escola de Instrutores - Design Instrucional</t>
+  </si>
+  <si>
+    <t>16 a 18/06/2026</t>
   </si>
   <si>
     <t>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T3</t>
@@ -8611,6 +8620,33 @@
     <t>André Pachioni Baeta</t>
   </si>
   <si>
+    <t>6371/2026</t>
+  </si>
+  <si>
+    <t>Painel MROSC</t>
+  </si>
+  <si>
+    <t>20/07/2026</t>
+  </si>
+  <si>
+    <t>6414/2026</t>
+  </si>
+  <si>
+    <t>31º SEMAT</t>
+  </si>
+  <si>
+    <t>3 e 4/08/2026</t>
+  </si>
+  <si>
+    <t>6503/2026</t>
+  </si>
+  <si>
+    <t>Curso “Sisaudit na Prática”</t>
+  </si>
+  <si>
+    <t>Davi Assunção Salvador Nery de Castro; David da Silva de Araújo; Hamilton de Jesus Lopes Neto</t>
+  </si>
+  <si>
     <t>ID Ação</t>
   </si>
   <si>
@@ -8755,6 +8791,9 @@
     <t>2026-042</t>
   </si>
   <si>
+    <t>2026-044</t>
+  </si>
+  <si>
     <t>DASHBOARD DE CURSOS — 2026</t>
   </si>
   <si>
@@ -8909,9 +8948,6 @@
   </si>
   <si>
     <t>Solicitado</t>
-  </si>
-  <si>
-    <t>Em andamento</t>
   </si>
   <si>
     <t>2026/2027</t>
@@ -8996,10 +9032,10 @@
     <t>Participantes</t>
   </si>
   <si>
-    <t>Escola de Instrutores - Design Instrucional</t>
-  </si>
-  <si>
-    <t>16 a 18/06/2026</t>
+    <t>teste</t>
+  </si>
+  <si>
+    <t>03/06/2026</t>
   </si>
 </sst>
 </file>
@@ -12229,10 +12265,10 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>13</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -12458,10 +12494,10 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>400</c:v>
+                  <c:v>417</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>371</c:v>
+                  <c:v>403</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>370</c:v>
@@ -12810,13 +12846,13 @@
                   <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -12911,7 +12947,7 @@
                 <c:formatCode>#,##0</c:formatCode>
                 <c:ptCount val="12"/>
                 <c:pt idx="0">
-                  <c:v>2</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -12935,7 +12971,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
@@ -14914,7 +14950,27 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1BD5F14-CD6F-4B62-85D2-128A9D3B5FF1}" name="Tabela2" displayName="Tabela2" ref="B1:T684" totalsRowShown="0" headerRowDxfId="50" dataDxfId="49" totalsRowDxfId="48" totalsRowBorderDxfId="47">
-  <autoFilter ref="B1:T684" xr:uid="{D1BD5F14-CD6F-4B62-85D2-128A9D3B5FF1}"/>
+  <autoFilter ref="B1:T684" xr:uid="{D1BD5F14-CD6F-4B62-85D2-128A9D3B5FF1}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
+    <filterColumn colId="12" hiddenButton="1"/>
+    <filterColumn colId="13" hiddenButton="1"/>
+    <filterColumn colId="14" hiddenButton="1"/>
+    <filterColumn colId="15" hiddenButton="1"/>
+    <filterColumn colId="16" hiddenButton="1"/>
+    <filterColumn colId="17" hiddenButton="1"/>
+    <filterColumn colId="18" hiddenButton="1"/>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:T684">
     <sortCondition ref="I1:I684"/>
   </sortState>
@@ -33822,7 +33878,7 @@
       <c r="S312" s="22">
         <v>75</v>
       </c>
-      <c r="T312" s="20" t="s">
+      <c r="T312" s="54" t="s">
         <v>1326</v>
       </c>
     </row>
@@ -38445,7 +38501,7 @@
         <v>0</v>
       </c>
       <c r="R386" s="23">
-        <f t="shared" ref="R386:R392" si="6">SUM(O386:Q386)</f>
+        <f t="shared" ref="R386:R449" si="6">SUM(O386:Q386)</f>
         <v>49</v>
       </c>
       <c r="S386" s="22">
@@ -50914,7 +50970,7 @@
         <v>30</v>
       </c>
       <c r="R586" s="23">
-        <f t="shared" ref="R586:R640" si="10">SUM(O586:Q586)</f>
+        <f t="shared" ref="R586:R649" si="10">SUM(O586:Q586)</f>
         <v>30</v>
       </c>
       <c r="S586" s="22">
@@ -56544,7 +56600,7 @@
         <v>2026</v>
       </c>
       <c r="C678" s="274" t="s">
-        <v>2748</v>
+        <v>21</v>
       </c>
       <c r="D678" s="64" t="s">
         <v>2749</v>
@@ -56573,16 +56629,24 @@
       <c r="L678" s="199">
         <v>16717.689999999999</v>
       </c>
-      <c r="M678" s="198"/>
+      <c r="M678" s="198">
+        <v>4.93</v>
+      </c>
       <c r="N678" s="62">
         <v>20</v>
       </c>
-      <c r="O678" s="63"/>
-      <c r="P678" s="63"/>
-      <c r="Q678" s="63"/>
+      <c r="O678" s="63">
+        <v>17</v>
+      </c>
+      <c r="P678" s="63">
+        <v>0</v>
+      </c>
+      <c r="Q678" s="63">
+        <v>0</v>
+      </c>
       <c r="R678" s="63">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="S678" s="64">
         <v>20</v>
@@ -56600,7 +56664,7 @@
         <v>2026</v>
       </c>
       <c r="C679" s="70" t="s">
-        <v>2748</v>
+        <v>21</v>
       </c>
       <c r="D679" s="180" t="s">
         <v>2753</v>
@@ -56629,14 +56693,24 @@
       <c r="L679" s="71">
         <v>9211.69</v>
       </c>
-      <c r="M679" s="197"/>
-      <c r="N679" s="184"/>
-      <c r="O679" s="185"/>
-      <c r="P679" s="185"/>
-      <c r="Q679" s="185"/>
+      <c r="M679" s="197">
+        <v>4.82</v>
+      </c>
+      <c r="N679" s="184">
+        <v>30</v>
+      </c>
+      <c r="O679" s="185">
+        <v>0</v>
+      </c>
+      <c r="P679" s="185">
+        <v>32</v>
+      </c>
+      <c r="Q679" s="185">
+        <v>0</v>
+      </c>
       <c r="R679" s="185">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="S679" s="180">
         <v>12</v>
@@ -56654,13 +56728,13 @@
         <v>2026</v>
       </c>
       <c r="C680" s="228" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D680" s="70" t="s">
         <v>2742</v>
       </c>
       <c r="E680" s="65" t="s">
-        <v>2942</v>
+        <v>2757</v>
       </c>
       <c r="F680" s="29" t="s">
         <v>23</v>
@@ -56669,7 +56743,7 @@
         <v>2693</v>
       </c>
       <c r="H680" s="68" t="s">
-        <v>2943</v>
+        <v>2758</v>
       </c>
       <c r="I680" s="69">
         <v>46189</v>
@@ -56714,7 +56788,7 @@
         <v>2753</v>
       </c>
       <c r="E681" s="273" t="s">
-        <v>2756</v>
+        <v>2759</v>
       </c>
       <c r="F681" s="31" t="s">
         <v>61</v>
@@ -56723,7 +56797,7 @@
         <v>2688</v>
       </c>
       <c r="H681" s="189" t="s">
-        <v>2757</v>
+        <v>2760</v>
       </c>
       <c r="I681" s="190">
         <v>46189</v>
@@ -56762,13 +56836,13 @@
         <v>2026</v>
       </c>
       <c r="C682" s="70" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D682" s="180" t="s">
-        <v>2758</v>
+        <v>2761</v>
       </c>
       <c r="E682" s="164" t="s">
-        <v>2759</v>
+        <v>2762</v>
       </c>
       <c r="F682" s="29" t="s">
         <v>61</v>
@@ -56777,7 +56851,7 @@
         <v>2688</v>
       </c>
       <c r="H682" s="182" t="s">
-        <v>2760</v>
+        <v>2763</v>
       </c>
       <c r="I682" s="183">
         <v>46195</v>
@@ -56816,13 +56890,13 @@
         <v>2026</v>
       </c>
       <c r="C683" s="70" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D683" s="186" t="s">
-        <v>2761</v>
+        <v>2764</v>
       </c>
       <c r="E683" s="187" t="s">
-        <v>2762</v>
+        <v>2765</v>
       </c>
       <c r="F683" s="31" t="s">
         <v>61</v>
@@ -56831,7 +56905,7 @@
         <v>71</v>
       </c>
       <c r="H683" s="189" t="s">
-        <v>2763</v>
+        <v>2766</v>
       </c>
       <c r="I683" s="190">
         <v>46335</v>
@@ -56870,13 +56944,13 @@
         <v>2026</v>
       </c>
       <c r="C684" s="228" t="s">
-        <v>2764</v>
+        <v>2767</v>
       </c>
       <c r="D684" s="70" t="s">
-        <v>2765</v>
+        <v>2768</v>
       </c>
       <c r="E684" s="164" t="s">
-        <v>2766</v>
+        <v>2769</v>
       </c>
       <c r="F684" s="66" t="s">
         <v>80</v>
@@ -56908,7 +56982,7 @@
         <v>32</v>
       </c>
       <c r="T684" s="67" t="s">
-        <v>2767</v>
+        <v>2770</v>
       </c>
     </row>
     <row r="685" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -56920,13 +56994,13 @@
         <v>2026</v>
       </c>
       <c r="C685" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D685" s="210" t="s">
-        <v>2768</v>
+        <v>2771</v>
       </c>
       <c r="E685" s="211" t="s">
-        <v>2769</v>
+        <v>2772</v>
       </c>
       <c r="F685" s="212" t="s">
         <v>61</v>
@@ -56935,7 +57009,7 @@
         <v>71</v>
       </c>
       <c r="H685" s="213" t="s">
-        <v>2770</v>
+        <v>2773</v>
       </c>
       <c r="I685" s="214">
         <v>46286</v>
@@ -56975,13 +57049,13 @@
         <v>2026</v>
       </c>
       <c r="C686" s="219" t="s">
-        <v>2764</v>
+        <v>2767</v>
       </c>
       <c r="D686" s="219" t="s">
-        <v>2771</v>
+        <v>2774</v>
       </c>
       <c r="E686" s="240" t="s">
-        <v>2772</v>
+        <v>2775</v>
       </c>
       <c r="F686" s="221" t="s">
         <v>23</v>
@@ -56990,7 +57064,7 @@
         <v>67</v>
       </c>
       <c r="H686" s="222" t="s">
-        <v>2773</v>
+        <v>2776</v>
       </c>
       <c r="I686" s="223">
         <v>46167</v>
@@ -57035,10 +57109,10 @@
         <v>2741</v>
       </c>
       <c r="D687" s="210" t="s">
-        <v>2774</v>
+        <v>2777</v>
       </c>
       <c r="E687" s="211" t="s">
-        <v>2775</v>
+        <v>2778</v>
       </c>
       <c r="F687" s="212" t="s">
         <v>23</v>
@@ -57047,7 +57121,7 @@
         <v>67</v>
       </c>
       <c r="H687" s="213" t="s">
-        <v>2776</v>
+        <v>2779</v>
       </c>
       <c r="I687" s="214">
         <v>46174</v>
@@ -57074,7 +57148,7 @@
         <v>25</v>
       </c>
       <c r="T687" t="s">
-        <v>2777</v>
+        <v>2780</v>
       </c>
       <c r="U687" s="203"/>
     </row>
@@ -57087,13 +57161,13 @@
         <v>2026</v>
       </c>
       <c r="C688" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D688" s="219" t="s">
-        <v>2778</v>
+        <v>2781</v>
       </c>
       <c r="E688" s="240" t="s">
-        <v>2779</v>
+        <v>2782</v>
       </c>
       <c r="F688" s="221" t="s">
         <v>80</v>
@@ -57102,7 +57176,7 @@
         <v>2725</v>
       </c>
       <c r="H688" s="222" t="s">
-        <v>2780</v>
+        <v>2783</v>
       </c>
       <c r="I688" s="223">
         <v>46204</v>
@@ -57147,10 +57221,10 @@
         <v>21</v>
       </c>
       <c r="D689" s="210" t="s">
-        <v>2781</v>
+        <v>2784</v>
       </c>
       <c r="E689" s="245" t="s">
-        <v>2782</v>
+        <v>2785</v>
       </c>
       <c r="F689" s="212" t="s">
         <v>23</v>
@@ -57159,7 +57233,7 @@
         <v>2709</v>
       </c>
       <c r="H689" s="247" t="s">
-        <v>2783</v>
+        <v>2786</v>
       </c>
       <c r="I689" s="214">
         <v>46154</v>
@@ -57171,7 +57245,7 @@
         <v>34</v>
       </c>
       <c r="L689" s="26">
-        <v>9067.76</v>
+        <v>6497.28</v>
       </c>
       <c r="M689" s="215">
         <v>4.88</v>
@@ -57209,13 +57283,13 @@
         <v>2026</v>
       </c>
       <c r="C690" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D690" s="219" t="s">
-        <v>2781</v>
+        <v>2784</v>
       </c>
       <c r="E690" s="246" t="s">
-        <v>2784</v>
+        <v>2787</v>
       </c>
       <c r="F690" s="221" t="s">
         <v>23</v>
@@ -57224,7 +57298,7 @@
         <v>2709</v>
       </c>
       <c r="H690" s="248" t="s">
-        <v>2785</v>
+        <v>2788</v>
       </c>
       <c r="I690" s="223">
         <v>46196</v>
@@ -57236,7 +57310,7 @@
         <v>34</v>
       </c>
       <c r="L690" s="26">
-        <v>9067.76</v>
+        <v>6497.28</v>
       </c>
       <c r="M690" s="215"/>
       <c r="N690" s="226">
@@ -57269,7 +57343,7 @@
         <v>21</v>
       </c>
       <c r="D691" s="210" t="s">
-        <v>2786</v>
+        <v>2789</v>
       </c>
       <c r="E691" s="245" t="s">
         <v>2667</v>
@@ -57281,7 +57355,7 @@
         <v>37</v>
       </c>
       <c r="H691" s="213" t="s">
-        <v>2787</v>
+        <v>2790</v>
       </c>
       <c r="I691" s="214">
         <v>46160</v>
@@ -57334,10 +57408,10 @@
         <v>21</v>
       </c>
       <c r="D692" s="219" t="s">
-        <v>2788</v>
+        <v>2791</v>
       </c>
       <c r="E692" s="246" t="s">
-        <v>2789</v>
+        <v>2792</v>
       </c>
       <c r="F692" s="221" t="s">
         <v>23</v>
@@ -57346,7 +57420,7 @@
         <v>363</v>
       </c>
       <c r="H692" s="222" t="s">
-        <v>2790</v>
+        <v>2793</v>
       </c>
       <c r="I692" s="223">
         <v>46140</v>
@@ -57399,10 +57473,10 @@
         <v>21</v>
       </c>
       <c r="D693" s="210" t="s">
-        <v>2791</v>
+        <v>2794</v>
       </c>
       <c r="E693" s="245" t="s">
-        <v>2792</v>
+        <v>2795</v>
       </c>
       <c r="F693" s="212" t="s">
         <v>23</v>
@@ -57411,7 +57485,7 @@
         <v>24</v>
       </c>
       <c r="H693" s="213" t="s">
-        <v>2793</v>
+        <v>2796</v>
       </c>
       <c r="I693" s="214">
         <v>46148</v>
@@ -57448,7 +57522,7 @@
         <v>12</v>
       </c>
       <c r="T693" s="209" t="s">
-        <v>2794</v>
+        <v>2797</v>
       </c>
       <c r="U693" s="203"/>
     </row>
@@ -57461,13 +57535,13 @@
         <v>2026</v>
       </c>
       <c r="C694" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D694" s="219" t="s">
-        <v>2795</v>
+        <v>2798</v>
       </c>
       <c r="E694" s="220" t="s">
-        <v>2796</v>
+        <v>2799</v>
       </c>
       <c r="F694" s="221" t="s">
         <v>61</v>
@@ -57476,7 +57550,7 @@
         <v>2688</v>
       </c>
       <c r="H694" s="222" t="s">
-        <v>2797</v>
+        <v>2800</v>
       </c>
       <c r="I694" s="223">
         <v>46157</v>
@@ -57514,13 +57588,13 @@
         <v>2026</v>
       </c>
       <c r="C695" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D695" s="210" t="s">
-        <v>2798</v>
+        <v>2801</v>
       </c>
       <c r="E695" s="211" t="s">
-        <v>2799</v>
+        <v>2802</v>
       </c>
       <c r="F695" s="212" t="s">
         <v>80</v>
@@ -57529,7 +57603,7 @@
         <v>2725</v>
       </c>
       <c r="H695" s="213" t="s">
-        <v>2800</v>
+        <v>2803</v>
       </c>
       <c r="I695" s="214">
         <v>46223</v>
@@ -57570,10 +57644,10 @@
         <v>21</v>
       </c>
       <c r="D696" s="219" t="s">
-        <v>2801</v>
+        <v>2804</v>
       </c>
       <c r="E696" s="220" t="s">
-        <v>2802</v>
+        <v>2805</v>
       </c>
       <c r="F696" s="221" t="s">
         <v>80</v>
@@ -57582,7 +57656,7 @@
         <v>2725</v>
       </c>
       <c r="H696" s="222" t="s">
-        <v>2803</v>
+        <v>2806</v>
       </c>
       <c r="I696" s="223">
         <v>46167</v>
@@ -57627,10 +57701,10 @@
         <v>21</v>
       </c>
       <c r="D697" s="210" t="s">
-        <v>2804</v>
+        <v>2807</v>
       </c>
       <c r="E697" s="211" t="s">
-        <v>2805</v>
+        <v>2808</v>
       </c>
       <c r="F697" s="212" t="s">
         <v>80</v>
@@ -57639,7 +57713,7 @@
         <v>2725</v>
       </c>
       <c r="H697" s="213" t="s">
-        <v>2806</v>
+        <v>2809</v>
       </c>
       <c r="I697" s="214">
         <v>46148</v>
@@ -57672,7 +57746,7 @@
         <v>3</v>
       </c>
       <c r="T697" s="209" t="s">
-        <v>2807</v>
+        <v>2810</v>
       </c>
       <c r="U697" s="203"/>
     </row>
@@ -57685,13 +57759,13 @@
         <v>2026</v>
       </c>
       <c r="C698" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D698" s="219" t="s">
-        <v>2808</v>
+        <v>2811</v>
       </c>
       <c r="E698" s="220" t="s">
-        <v>2809</v>
+        <v>2812</v>
       </c>
       <c r="F698" s="221" t="s">
         <v>23</v>
@@ -57700,7 +57774,7 @@
         <v>24</v>
       </c>
       <c r="H698" s="222" t="s">
-        <v>2797</v>
+        <v>2800</v>
       </c>
       <c r="I698" s="223">
         <v>46204</v>
@@ -57738,13 +57812,13 @@
         <v>2026</v>
       </c>
       <c r="C699" s="219" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
       <c r="D699" s="210" t="s">
-        <v>2810</v>
+        <v>2813</v>
       </c>
       <c r="E699" s="211" t="s">
-        <v>2811</v>
+        <v>2814</v>
       </c>
       <c r="F699" s="212" t="s">
         <v>23</v>
@@ -57753,7 +57827,7 @@
         <v>67</v>
       </c>
       <c r="H699" s="213" t="s">
-        <v>2812</v>
+        <v>2815</v>
       </c>
       <c r="I699" s="214">
         <v>46244</v>
@@ -57780,121 +57854,215 @@
         <v>10</v>
       </c>
       <c r="T699" s="209" t="s">
-        <v>2813</v>
+        <v>2816</v>
       </c>
       <c r="U699" s="203"/>
     </row>
     <row r="700" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A700" s="218" t="str">
         <f>IF(B700="","",B700&amp;"-"&amp;TEXT(COUNTIF(B$2:B700,B700),"000"))</f>
-        <v/>
-      </c>
-      <c r="B700" s="219"/>
-      <c r="C700" s="219"/>
-      <c r="D700" s="219"/>
-      <c r="E700" s="220"/>
-      <c r="F700" s="221"/>
-      <c r="G700" s="218"/>
-      <c r="H700" s="222"/>
-      <c r="I700" s="223"/>
-      <c r="J700" s="223"/>
-      <c r="K700" s="219"/>
-      <c r="L700" s="224"/>
+        <v>2026-044</v>
+      </c>
+      <c r="B700" s="219">
+        <v>2026</v>
+      </c>
+      <c r="C700" s="219" t="s">
+        <v>2756</v>
+      </c>
+      <c r="D700" s="219" t="s">
+        <v>2817</v>
+      </c>
+      <c r="E700" s="220" t="s">
+        <v>2818</v>
+      </c>
+      <c r="F700" s="221" t="s">
+        <v>61</v>
+      </c>
+      <c r="G700" s="218" t="s">
+        <v>71</v>
+      </c>
+      <c r="H700" s="222" t="s">
+        <v>2819</v>
+      </c>
+      <c r="I700" s="223">
+        <v>46223</v>
+      </c>
+      <c r="J700" s="223">
+        <v>46223</v>
+      </c>
+      <c r="K700" s="219" t="s">
+        <v>34</v>
+      </c>
+      <c r="L700" s="224">
+        <v>0</v>
+      </c>
       <c r="M700" s="215"/>
       <c r="N700" s="226"/>
       <c r="O700" s="225"/>
       <c r="P700" s="225"/>
       <c r="Q700" s="225"/>
-      <c r="R700" s="225" t="str">
+      <c r="R700" s="225">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="S700" s="219"/>
-      <c r="T700" s="218"/>
+        <v>0</v>
+      </c>
+      <c r="S700" s="219">
+        <v>4</v>
+      </c>
+      <c r="T700" s="218" t="s">
+        <v>471</v>
+      </c>
       <c r="U700" s="203"/>
     </row>
     <row r="701" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A701" s="209" t="str">
         <f>IF(B701="","",B701&amp;"-"&amp;TEXT(COUNTIF(B$2:B701,B701),"000"))</f>
-        <v/>
-      </c>
-      <c r="B701" s="210"/>
-      <c r="C701" s="219"/>
-      <c r="D701" s="210"/>
-      <c r="E701" s="211"/>
-      <c r="F701" s="212"/>
-      <c r="G701" s="209"/>
-      <c r="H701" s="213"/>
-      <c r="I701" s="214"/>
-      <c r="J701" s="214"/>
-      <c r="K701" s="210"/>
+        <v>2026-045</v>
+      </c>
+      <c r="B701" s="210">
+        <v>2026</v>
+      </c>
+      <c r="C701" s="219" t="s">
+        <v>2756</v>
+      </c>
+      <c r="D701" s="210" t="s">
+        <v>2820</v>
+      </c>
+      <c r="E701" s="211" t="s">
+        <v>2821</v>
+      </c>
+      <c r="F701" s="212" t="s">
+        <v>61</v>
+      </c>
+      <c r="G701" s="209" t="s">
+        <v>71</v>
+      </c>
+      <c r="H701" s="213" t="s">
+        <v>2822</v>
+      </c>
+      <c r="I701" s="214">
+        <v>46237</v>
+      </c>
+      <c r="J701" s="214">
+        <v>46238</v>
+      </c>
+      <c r="K701" s="210" t="s">
+        <v>34</v>
+      </c>
       <c r="L701" s="224"/>
       <c r="M701" s="215"/>
-      <c r="N701" s="216"/>
+      <c r="N701" s="216">
+        <v>400</v>
+      </c>
       <c r="O701" s="217"/>
       <c r="P701" s="217"/>
       <c r="Q701" s="217"/>
-      <c r="R701" s="217" t="str">
+      <c r="R701" s="217">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="S701" s="210"/>
+        <v>0</v>
+      </c>
+      <c r="S701" s="210">
+        <v>8</v>
+      </c>
       <c r="T701" s="209"/>
       <c r="U701" s="203"/>
     </row>
     <row r="702" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A702" s="218" t="str">
         <f>IF(B702="","",B702&amp;"-"&amp;TEXT(COUNTIF(B$2:B702,B702),"000"))</f>
-        <v/>
-      </c>
-      <c r="B702" s="219"/>
-      <c r="C702" s="219"/>
-      <c r="D702" s="219"/>
-      <c r="E702" s="220"/>
-      <c r="F702" s="221"/>
-      <c r="G702" s="218"/>
-      <c r="H702" s="222"/>
-      <c r="I702" s="223"/>
-      <c r="J702" s="223"/>
-      <c r="K702" s="219"/>
+        <v>2026-046</v>
+      </c>
+      <c r="B702" s="219">
+        <v>2026</v>
+      </c>
+      <c r="C702" s="219" t="s">
+        <v>2748</v>
+      </c>
+      <c r="D702" s="219" t="s">
+        <v>2823</v>
+      </c>
+      <c r="E702" s="220" t="s">
+        <v>2824</v>
+      </c>
+      <c r="F702" s="221" t="s">
+        <v>23</v>
+      </c>
+      <c r="G702" s="218" t="s">
+        <v>24</v>
+      </c>
+      <c r="H702" s="222" t="s">
+        <v>2758</v>
+      </c>
+      <c r="I702" s="223">
+        <v>46189</v>
+      </c>
+      <c r="J702" s="223">
+        <v>46191</v>
+      </c>
+      <c r="K702" s="219" t="s">
+        <v>34</v>
+      </c>
       <c r="L702" s="224"/>
       <c r="M702" s="215"/>
       <c r="N702" s="226"/>
       <c r="O702" s="225"/>
       <c r="P702" s="225"/>
       <c r="Q702" s="225"/>
-      <c r="R702" s="225" t="str">
+      <c r="R702" s="225">
         <f t="shared" si="14"/>
-        <v/>
-      </c>
-      <c r="S702" s="219"/>
-      <c r="T702" s="218"/>
+        <v>0</v>
+      </c>
+      <c r="S702" s="219">
+        <v>12</v>
+      </c>
+      <c r="T702" s="218" t="s">
+        <v>2825</v>
+      </c>
       <c r="U702" s="203"/>
     </row>
     <row r="703" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A703" s="209" t="str">
         <f>IF(B703="","",B703&amp;"-"&amp;TEXT(COUNTIF(B$2:B703,B703),"000"))</f>
-        <v/>
-      </c>
-      <c r="B703" s="210"/>
-      <c r="C703" s="219"/>
+        <v>2026-047</v>
+      </c>
+      <c r="B703" s="210">
+        <v>2026</v>
+      </c>
+      <c r="C703" s="219" t="s">
+        <v>2756</v>
+      </c>
       <c r="D703" s="210"/>
-      <c r="E703" s="211"/>
-      <c r="F703" s="212"/>
-      <c r="G703" s="209"/>
-      <c r="H703" s="213"/>
-      <c r="I703" s="214"/>
-      <c r="J703" s="214"/>
-      <c r="K703" s="210"/>
-      <c r="L703" s="224"/>
+      <c r="E703" s="211" t="s">
+        <v>2954</v>
+      </c>
+      <c r="F703" s="212" t="s">
+        <v>23</v>
+      </c>
+      <c r="G703" s="209" t="s">
+        <v>24</v>
+      </c>
+      <c r="H703" s="213" t="s">
+        <v>2955</v>
+      </c>
+      <c r="I703" s="213" t="s">
+        <v>2955</v>
+      </c>
+      <c r="J703" s="213" t="s">
+        <v>2955</v>
+      </c>
+      <c r="K703" s="210" t="s">
+        <v>34</v>
+      </c>
+      <c r="L703" s="224">
+        <v>1000</v>
+      </c>
       <c r="M703" s="215"/>
       <c r="N703" s="216"/>
       <c r="O703" s="217"/>
       <c r="P703" s="217"/>
       <c r="Q703" s="217"/>
-      <c r="R703" s="217" t="str">
+      <c r="R703" s="217">
         <f t="shared" si="14"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="S703" s="210"/>
       <c r="T703" s="209"/>
@@ -59229,6 +59397,7 @@
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <autoFilter ref="A1:A748" xr:uid="{9A950031-0FEE-4C02-A480-D14B9CA90666}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:T676">
     <sortCondition ref="B2:B676"/>
   </sortState>
@@ -59289,7 +59458,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Clique e insira um valor de a lista de itens" sqref="F518" xr:uid="{04F4F39B-F406-4ECC-A64A-F7A18A81A48D}">
       <formula1>"Interno,Externo,Híbrido"</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Erro" error="Insira uma data válida. Formato: DD/MM/AAAA" sqref="I594:J594 I647:J648 I658:J658 I662:J662 I664:I673 I644:J645 I596:J640 I573:J590 I463:J571 I2:J460 I676:J676 J664:J674 I681:J1048576" xr:uid="{A71E4390-A059-418C-8F5C-AD2AF445253E}">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Erro" error="Insira uma data válida. Formato: DD/MM/AAAA" sqref="I594:J594 I647:J648 I658:J658 I662:J662 I664:I673 I644:J645 I596:J640 I573:J590 I463:J571 I2:J460 I676:J676 J664:J674 I681:J702 I704:J1048576" xr:uid="{A71E4390-A059-418C-8F5C-AD2AF445253E}">
       <formula1>41640</formula1>
       <formula2>47848</formula2>
     </dataValidation>
@@ -59378,55 +59547,55 @@
         <v>1</v>
       </c>
       <c r="B1" s="96" t="s">
-        <v>2814</v>
+        <v>2826</v>
       </c>
       <c r="C1" s="96" t="s">
-        <v>2815</v>
+        <v>2827</v>
       </c>
       <c r="D1" s="96" t="s">
         <v>4</v>
       </c>
       <c r="E1" s="96" t="s">
-        <v>2816</v>
+        <v>2828</v>
       </c>
       <c r="F1" s="96" t="s">
         <v>19</v>
       </c>
       <c r="G1" s="96" t="s">
-        <v>2817</v>
+        <v>2829</v>
       </c>
       <c r="H1" s="96" t="s">
-        <v>2818</v>
+        <v>2830</v>
       </c>
       <c r="I1" s="96" t="s">
-        <v>2819</v>
+        <v>2831</v>
       </c>
       <c r="J1" s="96" t="s">
-        <v>2820</v>
+        <v>2832</v>
       </c>
       <c r="L1" s="129" t="s">
-        <v>2821</v>
+        <v>2833</v>
       </c>
       <c r="M1" s="100">
         <v>2026</v>
       </c>
       <c r="U1" s="162" t="s">
-        <v>2822</v>
+        <v>2834</v>
       </c>
       <c r="V1" s="161"/>
       <c r="X1" s="159" t="s">
-        <v>2823</v>
+        <v>2835</v>
       </c>
       <c r="Y1" s="107"/>
       <c r="Z1" s="107"/>
       <c r="AA1" s="107"/>
       <c r="AC1" s="254" t="s">
-        <v>2824</v>
+        <v>2836</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="98" cm="1">
-        <f t="array" ref="A2:J64">_xlfn.LET(_xlpm.totalRows,MAX(S4:S200),_xlpm.seq,_xlfn.SEQUENCE(_xlpm.totalRows),_xlpm.srcRow,_xlfn.MAP(_xlpm.seq,_xlfn.LAMBDA(_xlpm.s,MATCH(_xlpm.s-1,T4:T200,1))),_xlpm.instrIdx,_xlfn.MAP(_xlpm.seq,_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.s,_xlpm.sr,_xlpm.s-INDEX(T4:T200,_xlpm.sr))),_xlpm.ano,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(L4:L200,_xlpm.sr))),_xlpm.id,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(M4:M200,_xlpm.sr))),_xlpm.status,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(N4:N200,_xlpm.sr))),_xlpm.curso,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(O4:O200,_xlpm.sr))),_xlpm.ch,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(P4:P200,_xlpm.sr)+0)),_xlpm.instrStr,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(Q4:Q200,_xlpm.sr))),_xlpm.nInstr,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(R4:R200,_xlpm.sr)+0)),_xlpm.instrName,_xlfn.MAP(_xlpm.instrStr,_xlpm.instrIdx,_xlfn.LAMBDA(_xlpm.s,_xlpm.idx,TRIM(INDEX(_xlfn.TEXTSPLIT(_xlpm.s,"; "),,_xlpm.idx)))),_xlpm.ovKey,X3:X200&amp;"|"&amp;Y3:Y200,_xlpm.lookupKey,_xlpm.id&amp;"|"&amp;_xlpm.instrName,_xlpm.ovAula,_xlfn.MAP(_xlpm.lookupKey,_xlfn.LAMBDA(_xlpm.k,IFERROR(_xlfn.XLOOKUP(_xlpm.k,_xlpm.ovKey,Z3:Z200),""))),_xlpm.ovMat,_xlfn.MAP(_xlpm.lookupKey,_xlfn.LAMBDA(_xlpm.k,IFERROR(_xlfn.XLOOKUP(_xlpm.k,_xlpm.ovKey,AA3:AA200),""))),_xlpm.geccAula,_xlfn.MAP(_xlpm.ovAula,_xlpm.ch,_xlfn.LAMBDA(_xlpm.ov,_xlpm.c,IF(_xlpm.ov&lt;&gt;"",_xlpm.ov+0,_xlpm.c))),_xlpm.geccMat,_xlfn.MAP(_xlpm.ovMat,_xlpm.ch,_xlpm.nInstr,_xlfn.LAMBDA(_xlpm.ov,_xlpm.c,_xlpm.n,IF(_xlpm.ov&lt;&gt;"",_xlpm.ov+0,_xlpm.c*0.3/_xlpm.n))),_xlpm.geccTotal,_xlpm.geccAula+_xlpm.geccMat,_xlfn.HSTACK(_xlpm.ano,_xlpm.id,_xlpm.status,_xlpm.curso,_xlpm.ch,_xlpm.instrName,_xlpm.nInstr,_xlpm.geccAula,_xlpm.geccMat,_xlpm.geccTotal))</f>
+        <f t="array" ref="A2:J70">_xlfn.LET(_xlpm.totalRows,MAX(S4:S200),_xlpm.seq,_xlfn.SEQUENCE(_xlpm.totalRows),_xlpm.srcRow,_xlfn.MAP(_xlpm.seq,_xlfn.LAMBDA(_xlpm.s,MATCH(_xlpm.s-1,T4:T200,1))),_xlpm.instrIdx,_xlfn.MAP(_xlpm.seq,_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.s,_xlpm.sr,_xlpm.s-INDEX(T4:T200,_xlpm.sr))),_xlpm.ano,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(L4:L200,_xlpm.sr))),_xlpm.id,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(M4:M200,_xlpm.sr))),_xlpm.status,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(N4:N200,_xlpm.sr))),_xlpm.curso,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(O4:O200,_xlpm.sr))),_xlpm.ch,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(P4:P200,_xlpm.sr)+0)),_xlpm.instrStr,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(Q4:Q200,_xlpm.sr))),_xlpm.nInstr,_xlfn.MAP(_xlpm.srcRow,_xlfn.LAMBDA(_xlpm.sr,INDEX(R4:R200,_xlpm.sr)+0)),_xlpm.instrName,_xlfn.MAP(_xlpm.instrStr,_xlpm.instrIdx,_xlfn.LAMBDA(_xlpm.s,_xlpm.idx,TRIM(INDEX(_xlfn.TEXTSPLIT(_xlpm.s,"; "),,_xlpm.idx)))),_xlpm.ovKey,X3:X200&amp;"|"&amp;Y3:Y200,_xlpm.lookupKey,_xlpm.id&amp;"|"&amp;_xlpm.instrName,_xlpm.ovAula,_xlfn.MAP(_xlpm.lookupKey,_xlfn.LAMBDA(_xlpm.k,IFERROR(_xlfn.XLOOKUP(_xlpm.k,_xlpm.ovKey,Z3:Z200),""))),_xlpm.ovMat,_xlfn.MAP(_xlpm.lookupKey,_xlfn.LAMBDA(_xlpm.k,IFERROR(_xlfn.XLOOKUP(_xlpm.k,_xlpm.ovKey,AA3:AA200),""))),_xlpm.geccAula,_xlfn.MAP(_xlpm.ovAula,_xlpm.ch,_xlfn.LAMBDA(_xlpm.ov,_xlpm.c,IF(_xlpm.ov&lt;&gt;"",_xlpm.ov+0,_xlpm.c))),_xlpm.geccMat,_xlfn.MAP(_xlpm.ovMat,_xlpm.ch,_xlpm.nInstr,_xlfn.LAMBDA(_xlpm.ov,_xlpm.c,_xlpm.n,IF(_xlpm.ov&lt;&gt;"",_xlpm.ov+0,_xlpm.c*0.3/_xlpm.n))),_xlpm.geccTotal,_xlpm.geccAula+_xlpm.geccMat,_xlfn.HSTACK(_xlpm.ano,_xlpm.id,_xlpm.status,_xlpm.curso,_xlpm.ch,_xlpm.instrName,_xlpm.nInstr,_xlpm.geccAula,_xlpm.geccMat,_xlpm.geccTotal))</f>
         <v>2026</v>
       </c>
       <c r="B2" s="98" t="str">
@@ -59457,25 +59626,25 @@
         <v>10.4</v>
       </c>
       <c r="X2" s="160" t="s">
-        <v>2814</v>
+        <v>2826</v>
       </c>
       <c r="Y2" s="160" t="s">
         <v>19</v>
       </c>
       <c r="Z2" s="160" t="s">
-        <v>2825</v>
+        <v>2837</v>
       </c>
       <c r="AA2" s="160" t="s">
-        <v>2826</v>
+        <v>2838</v>
       </c>
       <c r="AC2" s="255" t="s">
         <v>1</v>
       </c>
       <c r="AD2" s="255" t="s">
-        <v>2827</v>
+        <v>2839</v>
       </c>
       <c r="AE2" s="255" t="s">
-        <v>2828</v>
+        <v>2840</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
@@ -59510,34 +59679,34 @@
         <v>5.2</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>2829</v>
+        <v>2841</v>
       </c>
       <c r="M3" s="19" t="s">
-        <v>2830</v>
+        <v>2842</v>
       </c>
       <c r="N3" s="19" t="s">
-        <v>2831</v>
+        <v>2843</v>
       </c>
       <c r="O3" s="19" t="s">
-        <v>2832</v>
+        <v>2844</v>
       </c>
       <c r="P3" s="19" t="s">
-        <v>2833</v>
+        <v>2845</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>2834</v>
+        <v>2846</v>
       </c>
       <c r="R3" s="19" t="s">
-        <v>2835</v>
+        <v>2847</v>
       </c>
       <c r="S3" s="19" t="s">
-        <v>2836</v>
+        <v>2848</v>
       </c>
       <c r="T3" s="19" t="s">
-        <v>2837</v>
+        <v>2849</v>
       </c>
       <c r="X3" t="s">
-        <v>2838</v>
+        <v>2850</v>
       </c>
       <c r="Y3" t="s">
         <v>2695</v>
@@ -59590,7 +59759,7 @@
         <v>5.2</v>
       </c>
       <c r="L4" cm="1">
-        <f t="array" ref="L4:Q35">_xlfn.LET(_xlpm.src,'Ações InCompany'!A2:T997,_xlpm.sAno,INDEX(_xlpm.src,,2),_xlpm.sMod,INDEX(_xlpm.src,,11),_xlfn._xlws.FILTER(_xlfn.HSTACK(INDEX(_xlpm.src,,2),INDEX(_xlpm.src,,1),INDEX(_xlpm.src,,3),INDEX(_xlpm.src,,5),INDEX(_xlpm.src,,19),INDEX(_xlpm.src,,20)),(_xlpm.sAno=M1)*(_xlpm.sMod="Instrutoria Interna"),""))</f>
+        <f t="array" ref="L4:Q39">_xlfn.LET(_xlpm.src,'Ações InCompany'!A2:T997,_xlpm.sAno,INDEX(_xlpm.src,,2),_xlpm.sMod,INDEX(_xlpm.src,,11),_xlfn._xlws.FILTER(_xlfn.HSTACK(INDEX(_xlpm.src,,2),INDEX(_xlpm.src,,1),INDEX(_xlpm.src,,3),INDEX(_xlpm.src,,5),INDEX(_xlpm.src,,19),INDEX(_xlpm.src,,20)),(_xlpm.sAno=M1)*(_xlpm.sMod="Instrutoria Interna"),""))</f>
         <v>2026</v>
       </c>
       <c r="M4" t="str">
@@ -59617,11 +59786,11 @@
         <v>1</v>
       </c>
       <c r="T4" cm="1">
-        <f t="array" ref="T4:T36">_xlfn.VSTACK(0,_xlfn._xlws.FILTER(S4:S200,S4:S200&lt;&gt;""))</f>
+        <f t="array" ref="T4:T40">_xlfn.VSTACK(0,_xlfn._xlws.FILTER(S4:S200,S4:S200&lt;&gt;""))</f>
         <v>0</v>
       </c>
       <c r="X4" t="s">
-        <v>2839</v>
+        <v>2851</v>
       </c>
       <c r="Y4" t="s">
         <v>2695</v>
@@ -59701,7 +59870,7 @@
         <v>1</v>
       </c>
       <c r="X5" t="s">
-        <v>2840</v>
+        <v>2852</v>
       </c>
       <c r="Y5" t="s">
         <v>2711</v>
@@ -59716,7 +59885,7 @@
         <v>2026</v>
       </c>
       <c r="AD5" s="95" t="s">
-        <v>2841</v>
+        <v>2853</v>
       </c>
       <c r="AE5" s="250">
         <v>16</v>
@@ -59781,10 +59950,10 @@
         <v>6</v>
       </c>
       <c r="X6" t="s">
-        <v>2840</v>
+        <v>2852</v>
       </c>
       <c r="Y6" t="s">
-        <v>2842</v>
+        <v>2854</v>
       </c>
       <c r="Z6">
         <v>1</v>
@@ -59796,7 +59965,7 @@
         <v>2026</v>
       </c>
       <c r="AD6" s="95" t="s">
-        <v>2843</v>
+        <v>2855</v>
       </c>
       <c r="AE6" s="250">
         <v>16</v>
@@ -59861,7 +60030,7 @@
         <v>8</v>
       </c>
       <c r="X7" s="98" t="s">
-        <v>2844</v>
+        <v>2856</v>
       </c>
       <c r="Y7" t="s">
         <v>2695</v>
@@ -59941,7 +60110,7 @@
         <v>9</v>
       </c>
       <c r="X8" t="s">
-        <v>2845</v>
+        <v>2857</v>
       </c>
       <c r="Y8" s="95" t="s">
         <v>1342</v>
@@ -60014,7 +60183,7 @@
         <v>11</v>
       </c>
       <c r="X9" t="s">
-        <v>2845</v>
+        <v>2857</v>
       </c>
       <c r="Y9" s="95" t="s">
         <v>1022</v>
@@ -60087,7 +60256,7 @@
         <v>12</v>
       </c>
       <c r="X10" t="s">
-        <v>2845</v>
+        <v>2857</v>
       </c>
       <c r="Y10" s="95" t="s">
         <v>1366</v>
@@ -60160,10 +60329,10 @@
         <v>14</v>
       </c>
       <c r="X11" t="s">
-        <v>2845</v>
+        <v>2857</v>
       </c>
       <c r="Y11" s="95" t="s">
-        <v>2846</v>
+        <v>2858</v>
       </c>
       <c r="AA11">
         <v>1.2</v>
@@ -60233,10 +60402,10 @@
         <v>15</v>
       </c>
       <c r="X12" t="s">
-        <v>2845</v>
+        <v>2857</v>
       </c>
       <c r="Y12" s="95" t="s">
-        <v>2847</v>
+        <v>2859</v>
       </c>
       <c r="AA12">
         <v>1.2</v>
@@ -60306,7 +60475,7 @@
         <v>16</v>
       </c>
       <c r="X13" t="s">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="Y13" s="95" t="s">
         <v>1342</v>
@@ -60379,7 +60548,7 @@
         <v>18</v>
       </c>
       <c r="X14" t="s">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="Y14" s="95" t="s">
         <v>1022</v>
@@ -60452,7 +60621,7 @@
         <v>20</v>
       </c>
       <c r="X15" t="s">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="Y15" s="95" t="s">
         <v>1366</v>
@@ -60525,10 +60694,10 @@
         <v>22</v>
       </c>
       <c r="X16" t="s">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="Y16" s="95" t="s">
-        <v>2846</v>
+        <v>2858</v>
       </c>
       <c r="AA16">
         <v>1.2</v>
@@ -60598,10 +60767,10 @@
         <v>23</v>
       </c>
       <c r="X17" t="s">
-        <v>2848</v>
+        <v>2860</v>
       </c>
       <c r="Y17" s="95" t="s">
-        <v>2847</v>
+        <v>2859</v>
       </c>
       <c r="AA17">
         <v>1.2</v>
@@ -60671,7 +60840,7 @@
         <v>28</v>
       </c>
       <c r="X18" t="s">
-        <v>2849</v>
+        <v>2861</v>
       </c>
       <c r="Y18" s="95" t="s">
         <v>1342</v>
@@ -60744,7 +60913,7 @@
         <v>33</v>
       </c>
       <c r="X19" t="s">
-        <v>2849</v>
+        <v>2861</v>
       </c>
       <c r="Y19" s="95" t="s">
         <v>1022</v>
@@ -60796,7 +60965,7 @@
         <v>2026-022</v>
       </c>
       <c r="N20" t="str">
-        <v>A realizar</v>
+        <v>Realizado</v>
       </c>
       <c r="O20" t="str">
         <v>Fiscalizações Baseadas em Risco</v>
@@ -60817,7 +60986,7 @@
         <v>34</v>
       </c>
       <c r="X20" t="s">
-        <v>2849</v>
+        <v>2861</v>
       </c>
       <c r="Y20" s="95" t="s">
         <v>1366</v>
@@ -60869,7 +61038,7 @@
         <v>2026-023</v>
       </c>
       <c r="N21" t="str">
-        <v>A realizar</v>
+        <v>Realizado</v>
       </c>
       <c r="O21" t="str">
         <v>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T2</v>
@@ -60890,10 +61059,10 @@
         <v>36</v>
       </c>
       <c r="X21" t="s">
-        <v>2849</v>
+        <v>2861</v>
       </c>
       <c r="Y21" s="95" t="s">
-        <v>2846</v>
+        <v>2858</v>
       </c>
       <c r="AA21">
         <v>1.2</v>
@@ -60963,10 +61132,10 @@
         <v>38</v>
       </c>
       <c r="X22" t="s">
-        <v>2849</v>
+        <v>2861</v>
       </c>
       <c r="Y22" s="95" t="s">
-        <v>2847</v>
+        <v>2859</v>
       </c>
       <c r="AA22">
         <v>1.2</v>
@@ -61015,7 +61184,7 @@
         <v>2026-025</v>
       </c>
       <c r="N23" t="str">
-        <v>A realizar</v>
+        <v>Em andamento</v>
       </c>
       <c r="O23" t="str">
         <v>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T3</v>
@@ -61036,7 +61205,7 @@
         <v>39</v>
       </c>
       <c r="X23" s="98" t="s">
-        <v>2850</v>
+        <v>2862</v>
       </c>
       <c r="Y23" s="95" t="s">
         <v>2711</v>
@@ -61109,10 +61278,10 @@
         <v>41</v>
       </c>
       <c r="X24" s="98" t="s">
-        <v>2850</v>
+        <v>2862</v>
       </c>
       <c r="Y24" s="95" t="s">
-        <v>2842</v>
+        <v>2854</v>
       </c>
       <c r="AA24">
         <v>0</v>
@@ -61182,7 +61351,7 @@
         <v>43</v>
       </c>
       <c r="X25" t="s">
-        <v>2851</v>
+        <v>2863</v>
       </c>
       <c r="Y25" s="95" t="s">
         <v>854</v>
@@ -61255,10 +61424,10 @@
         <v>45</v>
       </c>
       <c r="X26" t="s">
-        <v>2851</v>
+        <v>2863</v>
       </c>
       <c r="Y26" s="95" t="s">
-        <v>2852</v>
+        <v>2864</v>
       </c>
       <c r="Z26">
         <v>0</v>
@@ -61331,7 +61500,7 @@
         <v>47</v>
       </c>
       <c r="X27" s="257" t="s">
-        <v>2853</v>
+        <v>2865</v>
       </c>
       <c r="Y27" s="95" t="s">
         <v>2711</v>
@@ -61404,10 +61573,10 @@
         <v>49</v>
       </c>
       <c r="X28" s="257" t="s">
-        <v>2853</v>
+        <v>2865</v>
       </c>
       <c r="Y28" s="95" t="s">
-        <v>2842</v>
+        <v>2854</v>
       </c>
       <c r="AA28">
         <v>0</v>
@@ -61477,7 +61646,7 @@
         <v>50</v>
       </c>
       <c r="X29" s="257" t="s">
-        <v>2854</v>
+        <v>2866</v>
       </c>
       <c r="Y29" s="95" t="s">
         <v>2711</v>
@@ -61550,10 +61719,10 @@
         <v>51</v>
       </c>
       <c r="X30" s="257" t="s">
+        <v>2866</v>
+      </c>
+      <c r="Y30" s="95" t="s">
         <v>2854</v>
-      </c>
-      <c r="Y30" s="95" t="s">
-        <v>2842</v>
       </c>
       <c r="AA30">
         <v>0</v>
@@ -61623,7 +61792,7 @@
         <v>56</v>
       </c>
       <c r="X31" s="257" t="s">
-        <v>2855</v>
+        <v>2867</v>
       </c>
       <c r="Y31" s="95" t="s">
         <v>471</v>
@@ -61699,7 +61868,7 @@
         <v>58</v>
       </c>
       <c r="X32" s="257" t="s">
-        <v>2856</v>
+        <v>2868</v>
       </c>
       <c r="Y32" t="s">
         <v>1342</v>
@@ -61775,10 +61944,10 @@
         <v>59</v>
       </c>
       <c r="X33" s="257" t="s">
-        <v>2856</v>
+        <v>2868</v>
       </c>
       <c r="Y33" t="s">
-        <v>2857</v>
+        <v>2869</v>
       </c>
       <c r="Z33">
         <v>4</v>
@@ -61788,7 +61957,7 @@
       </c>
       <c r="AC33" s="251"/>
       <c r="AD33" s="252" t="s">
-        <v>2858</v>
+        <v>2870</v>
       </c>
       <c r="AE33" s="253">
         <f>SUM(AE3:AE32)</f>
@@ -61854,10 +62023,10 @@
         <v>60</v>
       </c>
       <c r="X34" s="257" t="s">
-        <v>2856</v>
+        <v>2868</v>
       </c>
       <c r="Y34" t="s">
-        <v>2859</v>
+        <v>2871</v>
       </c>
       <c r="Z34">
         <v>4</v>
@@ -61925,7 +62094,7 @@
         <v>62</v>
       </c>
       <c r="X35" s="257" t="s">
-        <v>2856</v>
+        <v>2868</v>
       </c>
       <c r="Y35" t="s">
         <v>107</v>
@@ -61945,7 +62114,7 @@
         <v>2026-022</v>
       </c>
       <c r="C36" s="98" t="str">
-        <v>A realizar</v>
+        <v>Realizado</v>
       </c>
       <c r="D36" s="95" t="str">
         <v>Fiscalizações Baseadas em Risco</v>
@@ -61968,17 +62137,35 @@
       <c r="J36" s="99">
         <v>23</v>
       </c>
-      <c r="R36" t="str">
-        <v/>
-      </c>
-      <c r="S36" t="str">
-        <v/>
+      <c r="L36">
+        <v>2026</v>
+      </c>
+      <c r="M36" t="str">
+        <v>2026-044</v>
+      </c>
+      <c r="N36" t="str">
+        <v>A realizar</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Painel MROSC</v>
+      </c>
+      <c r="P36">
+        <v>4</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>Diversos</v>
+      </c>
+      <c r="R36">
+        <v>1</v>
+      </c>
+      <c r="S36">
+        <v>64</v>
       </c>
       <c r="T36">
         <v>63</v>
       </c>
       <c r="X36" s="257" t="s">
-        <v>2856</v>
+        <v>2868</v>
       </c>
       <c r="Y36" t="s">
         <v>548</v>
@@ -61998,7 +62185,7 @@
         <v>2026-022</v>
       </c>
       <c r="C37" s="163" t="str">
-        <v>A realizar</v>
+        <v>Realizado</v>
       </c>
       <c r="D37" t="str">
         <v>Fiscalizações Baseadas em Risco</v>
@@ -62021,14 +62208,35 @@
       <c r="J37" s="163">
         <v>23</v>
       </c>
-      <c r="R37" t="str">
-        <v/>
-      </c>
-      <c r="S37" t="str">
-        <v/>
+      <c r="L37">
+        <v>2026</v>
+      </c>
+      <c r="M37" t="str">
+        <v>2026-045</v>
+      </c>
+      <c r="N37" t="str">
+        <v>A realizar</v>
+      </c>
+      <c r="O37" t="str">
+        <v>31º SEMAT</v>
+      </c>
+      <c r="P37">
+        <v>8</v>
+      </c>
+      <c r="Q37">
+        <v>0</v>
+      </c>
+      <c r="R37">
+        <v>1</v>
+      </c>
+      <c r="S37">
+        <v>65</v>
+      </c>
+      <c r="T37">
+        <v>64</v>
       </c>
       <c r="X37" t="s">
-        <v>2860</v>
+        <v>2872</v>
       </c>
       <c r="Y37" t="s">
         <v>417</v>
@@ -62048,7 +62256,7 @@
         <v>2026-023</v>
       </c>
       <c r="C38" s="163" t="str">
-        <v>A realizar</v>
+        <v>Realizado</v>
       </c>
       <c r="D38" t="str">
         <v>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T2</v>
@@ -62071,14 +62279,35 @@
       <c r="J38" s="163">
         <v>13.8</v>
       </c>
-      <c r="R38" t="str">
-        <v/>
-      </c>
-      <c r="S38" t="str">
-        <v/>
+      <c r="L38">
+        <v>2026</v>
+      </c>
+      <c r="M38" t="str">
+        <v>2026-046</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Em andamento</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Curso “Sisaudit na Prática”</v>
+      </c>
+      <c r="P38">
+        <v>12</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>Davi Assunção Salvador Nery de Castro; David da Silva de Araújo; Hamilton de Jesus Lopes Neto</v>
+      </c>
+      <c r="R38">
+        <v>3</v>
+      </c>
+      <c r="S38">
+        <v>68</v>
+      </c>
+      <c r="T38">
+        <v>65</v>
       </c>
       <c r="X38" t="s">
-        <v>2860</v>
+        <v>2872</v>
       </c>
       <c r="Y38" s="260" t="s">
         <v>1095</v>
@@ -62098,7 +62327,7 @@
         <v>2026-023</v>
       </c>
       <c r="C39" s="163" t="str">
-        <v>A realizar</v>
+        <v>Realizado</v>
       </c>
       <c r="D39" t="str">
         <v>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T2</v>
@@ -62121,14 +62350,35 @@
       <c r="J39" s="163">
         <v>13.8</v>
       </c>
-      <c r="R39" t="str">
-        <v/>
-      </c>
-      <c r="S39" t="str">
-        <v/>
+      <c r="L39">
+        <v>2026</v>
+      </c>
+      <c r="M39" t="str">
+        <v>2026-047</v>
+      </c>
+      <c r="N39" t="str">
+        <v>A realizar</v>
+      </c>
+      <c r="O39" t="str">
+        <v>teste</v>
+      </c>
+      <c r="P39">
+        <v>0</v>
+      </c>
+      <c r="Q39">
+        <v>0</v>
+      </c>
+      <c r="R39">
+        <v>1</v>
+      </c>
+      <c r="S39">
+        <v>69</v>
+      </c>
+      <c r="T39">
+        <v>68</v>
       </c>
       <c r="X39" t="s">
-        <v>2861</v>
+        <v>2873</v>
       </c>
       <c r="Y39" t="s">
         <v>548</v>
@@ -62177,6 +62427,21 @@
       <c r="S40" t="str">
         <v/>
       </c>
+      <c r="T40">
+        <v>69</v>
+      </c>
+      <c r="X40" t="s">
+        <v>2874</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>471</v>
+      </c>
+      <c r="Z40">
+        <v>0</v>
+      </c>
+      <c r="AA40">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A41">
@@ -62186,7 +62451,7 @@
         <v>2026-025</v>
       </c>
       <c r="C41" s="163" t="str">
-        <v>A realizar</v>
+        <v>Em andamento</v>
       </c>
       <c r="D41" t="str">
         <v>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T3</v>
@@ -62224,7 +62489,7 @@
         <v>2026-025</v>
       </c>
       <c r="C42" s="163" t="str">
-        <v>A realizar</v>
+        <v>Em andamento</v>
       </c>
       <c r="D42" t="str">
         <v>Curso de formação para gestores e fiscais de Contrato em equipamentos nas unidades hospitalares - T3</v>
@@ -63090,7 +63355,37 @@
         <v/>
       </c>
     </row>
-    <row r="65" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>2026</v>
+      </c>
+      <c r="B65" t="str">
+        <v>2026-044</v>
+      </c>
+      <c r="C65" t="str">
+        <v>A realizar</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Painel MROSC</v>
+      </c>
+      <c r="E65">
+        <v>4</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Diversos</v>
+      </c>
+      <c r="G65">
+        <v>1</v>
+      </c>
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65">
+        <v>0</v>
+      </c>
+      <c r="J65">
+        <v>0</v>
+      </c>
       <c r="R65" t="str">
         <v/>
       </c>
@@ -63098,7 +63393,37 @@
         <v/>
       </c>
     </row>
-    <row r="66" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>2026</v>
+      </c>
+      <c r="B66" t="str">
+        <v>2026-045</v>
+      </c>
+      <c r="C66" t="str">
+        <v>A realizar</v>
+      </c>
+      <c r="D66" t="str">
+        <v>31º SEMAT</v>
+      </c>
+      <c r="E66">
+        <v>8</v>
+      </c>
+      <c r="F66" t="str">
+        <v>0</v>
+      </c>
+      <c r="G66">
+        <v>1</v>
+      </c>
+      <c r="H66">
+        <v>8</v>
+      </c>
+      <c r="I66">
+        <v>2.4</v>
+      </c>
+      <c r="J66">
+        <v>10.4</v>
+      </c>
       <c r="R66" t="str">
         <v/>
       </c>
@@ -63106,7 +63431,37 @@
         <v/>
       </c>
     </row>
-    <row r="67" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>2026</v>
+      </c>
+      <c r="B67" t="str">
+        <v>2026-046</v>
+      </c>
+      <c r="C67" t="str">
+        <v>Em andamento</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Curso “Sisaudit na Prática”</v>
+      </c>
+      <c r="E67">
+        <v>12</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Davi Assunção Salvador Nery de Castro</v>
+      </c>
+      <c r="G67">
+        <v>3</v>
+      </c>
+      <c r="H67">
+        <v>12</v>
+      </c>
+      <c r="I67">
+        <v>1.2</v>
+      </c>
+      <c r="J67">
+        <v>13.2</v>
+      </c>
       <c r="R67" t="str">
         <v/>
       </c>
@@ -63114,7 +63469,37 @@
         <v/>
       </c>
     </row>
-    <row r="68" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>2026</v>
+      </c>
+      <c r="B68" t="str">
+        <v>2026-046</v>
+      </c>
+      <c r="C68" t="str">
+        <v>Em andamento</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Curso “Sisaudit na Prática”</v>
+      </c>
+      <c r="E68">
+        <v>12</v>
+      </c>
+      <c r="F68" t="str">
+        <v>David da Silva de Araújo</v>
+      </c>
+      <c r="G68">
+        <v>3</v>
+      </c>
+      <c r="H68">
+        <v>12</v>
+      </c>
+      <c r="I68">
+        <v>1.2</v>
+      </c>
+      <c r="J68">
+        <v>13.2</v>
+      </c>
       <c r="R68" t="str">
         <v/>
       </c>
@@ -63122,7 +63507,37 @@
         <v/>
       </c>
     </row>
-    <row r="69" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>2026</v>
+      </c>
+      <c r="B69" t="str">
+        <v>2026-046</v>
+      </c>
+      <c r="C69" t="str">
+        <v>Em andamento</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Curso “Sisaudit na Prática”</v>
+      </c>
+      <c r="E69">
+        <v>12</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Hamilton de Jesus Lopes Neto</v>
+      </c>
+      <c r="G69">
+        <v>3</v>
+      </c>
+      <c r="H69">
+        <v>12</v>
+      </c>
+      <c r="I69">
+        <v>1.2</v>
+      </c>
+      <c r="J69">
+        <v>13.2</v>
+      </c>
       <c r="R69" t="str">
         <v/>
       </c>
@@ -63130,7 +63545,37 @@
         <v/>
       </c>
     </row>
-    <row r="70" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>2026</v>
+      </c>
+      <c r="B70" t="str">
+        <v>2026-047</v>
+      </c>
+      <c r="C70" t="str">
+        <v>A realizar</v>
+      </c>
+      <c r="D70" t="str">
+        <v>teste</v>
+      </c>
+      <c r="E70">
+        <v>0</v>
+      </c>
+      <c r="F70" t="str">
+        <v>0</v>
+      </c>
+      <c r="G70">
+        <v>1</v>
+      </c>
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70">
+        <v>0</v>
+      </c>
+      <c r="J70">
+        <v>0</v>
+      </c>
       <c r="R70" t="str">
         <v/>
       </c>
@@ -63138,7 +63583,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R71" t="str">
         <v/>
       </c>
@@ -63146,7 +63591,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R72" t="str">
         <v/>
       </c>
@@ -63154,7 +63599,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R73" t="str">
         <v/>
       </c>
@@ -63162,7 +63607,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R74" t="str">
         <v/>
       </c>
@@ -63170,7 +63615,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R75" t="str">
         <v/>
       </c>
@@ -63178,7 +63623,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R76" t="str">
         <v/>
       </c>
@@ -63186,7 +63631,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R77" t="str">
         <v/>
       </c>
@@ -63194,7 +63639,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R78" t="str">
         <v/>
       </c>
@@ -63202,7 +63647,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R79" t="str">
         <v/>
       </c>
@@ -63210,7 +63655,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" spans="18:19" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:19" x14ac:dyDescent="0.25">
       <c r="R80" t="str">
         <v/>
       </c>
@@ -64201,7 +64646,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="50.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="280" t="s">
-        <v>2862</v>
+        <v>2875</v>
       </c>
       <c r="B1" s="280"/>
       <c r="C1" s="280"/>
@@ -64222,31 +64667,31 @@
     <row r="3" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="281" t="s">
-        <v>2863</v>
+        <v>2876</v>
       </c>
       <c r="B4" s="282"/>
       <c r="D4" s="283" t="s">
-        <v>2864</v>
+        <v>2877</v>
       </c>
       <c r="E4" s="284"/>
       <c r="G4" s="125" t="s">
-        <v>2865</v>
+        <v>2878</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="54.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
       <c r="A5" s="115">
         <f>COUNTIF('Ações InCompany'!B:B,2026)</f>
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B5" s="116" t="s">
-        <v>2866</v>
+        <v>2879</v>
       </c>
       <c r="D5" s="123">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado")</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E5" s="124" t="s">
-        <v>2866</v>
+        <v>2879</v>
       </c>
       <c r="G5" s="126">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"A realizar")</f>
@@ -64264,11 +64709,11 @@
     </row>
     <row r="8" spans="1:7" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A8" s="278" t="s">
-        <v>2867</v>
+        <v>2880</v>
       </c>
       <c r="B8" s="278"/>
       <c r="D8" s="278" t="s">
-        <v>2868</v>
+        <v>2881</v>
       </c>
       <c r="E8" s="278"/>
     </row>
@@ -64283,13 +64728,13 @@
         <v>5</v>
       </c>
       <c r="B10" s="108" t="s">
-        <v>2869</v>
+        <v>2882</v>
       </c>
       <c r="D10" s="108" t="s">
-        <v>2870</v>
+        <v>2883</v>
       </c>
       <c r="E10" s="108" t="s">
-        <v>2871</v>
+        <v>2884</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -64298,14 +64743,14 @@
       </c>
       <c r="B11" s="110">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado",'Ações InCompany'!F:F,"Servidores do TCDF")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D11" s="109" t="s">
-        <v>2872</v>
+        <v>2885</v>
       </c>
       <c r="E11" s="110">
         <f>SUMIFS('Ações InCompany'!O:O,'Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado")</f>
-        <v>400</v>
+        <v>417</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -64314,14 +64759,14 @@
       </c>
       <c r="B12" s="112">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado",'Ações InCompany'!F:F,"Jurisdicionados")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D12" s="111" t="s">
-        <v>2873</v>
+        <v>2886</v>
       </c>
       <c r="E12" s="112">
         <f>SUMIFS('Ações InCompany'!P:P,'Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado")</f>
-        <v>371</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
@@ -64333,7 +64778,7 @@
         <v>5</v>
       </c>
       <c r="D13" s="109" t="s">
-        <v>2874</v>
+        <v>2887</v>
       </c>
       <c r="E13" s="110">
         <f>SUMIFS('Ações InCompany'!Q:Q,'Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado")</f>
@@ -64342,23 +64787,23 @@
     </row>
     <row r="14" spans="1:7" ht="27.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="113" t="s">
-        <v>2875</v>
+        <v>2888</v>
       </c>
       <c r="B14" s="114">
         <f>SUM(B11:B13)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D14" s="113" t="s">
-        <v>2876</v>
+        <v>2889</v>
       </c>
       <c r="E14" s="114">
         <f>SUM(E11:E13)</f>
-        <v>1141</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A30" s="278" t="s">
-        <v>2877</v>
+        <v>2890</v>
       </c>
       <c r="B30" s="278"/>
       <c r="C30" s="278"/>
@@ -64377,16 +64822,16 @@
         <v>6</v>
       </c>
       <c r="B32" s="108" t="s">
-        <v>2878</v>
+        <v>2891</v>
       </c>
       <c r="C32" s="108" t="s">
-        <v>2879</v>
+        <v>2892</v>
       </c>
       <c r="D32" s="108" t="s">
-        <v>2880</v>
+        <v>2893</v>
       </c>
       <c r="E32" s="108" t="s">
-        <v>2881</v>
+        <v>2894</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64399,15 +64844,15 @@
       </c>
       <c r="C33" s="127">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"A realizar",'Ações InCompany'!G:G,A33)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D33" s="117">
         <f t="shared" ref="D33:D44" si="0">B33+C33</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E33" s="118">
         <f t="shared" ref="E33:E44" si="1">D33/$D$45</f>
-        <v>0.17948717948717949</v>
+        <v>0.21951219512195122</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64428,7 +64873,7 @@
       </c>
       <c r="E34" s="120">
         <f t="shared" si="1"/>
-        <v>7.6923076923076927E-2</v>
+        <v>7.3170731707317069E-2</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64449,7 +64894,7 @@
       </c>
       <c r="E35" s="118">
         <f t="shared" si="1"/>
-        <v>0.12820512820512819</v>
+        <v>0.12195121951219512</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64470,7 +64915,7 @@
       </c>
       <c r="E36" s="120">
         <f t="shared" si="1"/>
-        <v>5.128205128205128E-2</v>
+        <v>4.878048780487805E-2</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64491,7 +64936,7 @@
       </c>
       <c r="E37" s="118">
         <f t="shared" si="1"/>
-        <v>5.128205128205128E-2</v>
+        <v>4.878048780487805E-2</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64512,7 +64957,7 @@
       </c>
       <c r="E38" s="120">
         <f t="shared" si="1"/>
-        <v>0.17948717948717949</v>
+        <v>0.17073170731707318</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64521,7 +64966,7 @@
       </c>
       <c r="B39" s="145">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado",'Ações InCompany'!G:G,A39)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="146">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"A realizar",'Ações InCompany'!G:G,A39)</f>
@@ -64529,11 +64974,11 @@
       </c>
       <c r="D39" s="145">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E39" s="147">
         <f t="shared" si="1"/>
-        <v>7.6923076923076927E-2</v>
+        <v>9.7560975609756101E-2</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64554,7 +64999,7 @@
       </c>
       <c r="E40" s="158">
         <f>D40/$D$45</f>
-        <v>2.564102564102564E-2</v>
+        <v>2.4390243902439025E-2</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -64563,24 +65008,24 @@
       </c>
       <c r="B41" s="151">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado",'Ações InCompany'!G:G,A41)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C41" s="152">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"A realizar",'Ações InCompany'!G:G,A41)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D41" s="151">
         <f>B41+C41</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E41" s="157">
         <f>D41/$D$45</f>
-        <v>0.17948717948717949</v>
+        <v>0.14634146341463414</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="156" t="s">
-        <v>2882</v>
+        <v>2895</v>
       </c>
       <c r="B42" s="153">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado",'Ações InCompany'!G:G,A42)</f>
@@ -64617,12 +65062,12 @@
       </c>
       <c r="E43" s="157">
         <f>D43/$D$45</f>
-        <v>5.128205128205128E-2</v>
+        <v>4.878048780487805E-2</v>
       </c>
     </row>
     <row r="44" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="148" t="s">
-        <v>2883</v>
+        <v>2896</v>
       </c>
       <c r="B44" s="149">
         <f>COUNTIFS('Ações InCompany'!B:B,2026,'Ações InCompany'!C:C,"Realizado",'Ações InCompany'!G:G,"")</f>
@@ -64643,11 +65088,11 @@
     </row>
     <row r="45" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="113" t="s">
-        <v>2875</v>
+        <v>2888</v>
       </c>
       <c r="B45" s="121">
         <f>SUM(B33:B44)</f>
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C45" s="121">
         <f>SUM(C33:C44)</f>
@@ -64655,7 +65100,7 @@
       </c>
       <c r="D45" s="121">
         <f>SUM(D33:D44)</f>
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E45" s="122">
         <f>SUM(E33:E44)</f>
@@ -64694,163 +65139,163 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>2884</v>
+        <v>2897</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>2885</v>
+        <v>2898</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>2886</v>
+        <v>2899</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>2887</v>
+        <v>2900</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>2888</v>
+        <v>2901</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>1728</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>2891</v>
+        <v>2904</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>2892</v>
+        <v>2905</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C3" s="14" t="s">
         <v>24</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>2893</v>
+        <v>2906</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>2894</v>
+        <v>2907</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>67</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>2891</v>
+        <v>2904</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>2895</v>
+        <v>2908</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>71</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>2896</v>
+        <v>2909</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>2897</v>
+        <v>2910</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>2725</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>2898</v>
+        <v>2911</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>2899</v>
+        <v>2912</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>2900</v>
+        <v>2913</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>32</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>2901</v>
+        <v>2914</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>2902</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>2900</v>
+        <v>2913</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>2903</v>
+        <v>2916</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>2904</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>2905</v>
+        <v>2918</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>456</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>2906</v>
+        <v>2919</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>2907</v>
+        <v>2920</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>2905</v>
+        <v>2918</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>198</v>
@@ -64859,15 +65304,15 @@
         <v>23</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>2908</v>
+        <v>2921</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>2889</v>
+        <v>2902</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>2905</v>
+        <v>2918</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>363</v>
@@ -64876,7 +65321,7 @@
         <v>23</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>2909</v>
+        <v>2922</v>
       </c>
     </row>
   </sheetData>
@@ -64898,16 +65343,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="15" t="s">
-        <v>2910</v>
+        <v>2923</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>2911</v>
+        <v>2924</v>
       </c>
       <c r="D1" s="15" t="s">
-        <v>2815</v>
+        <v>2827</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -64918,10 +65363,10 @@
         <v>34</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>2912</v>
+        <v>2925</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>2748</v>
+        <v>2756</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -64932,10 +65377,10 @@
         <v>26</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>2913</v>
+        <v>2926</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>2914</v>
+        <v>2748</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -64959,7 +65404,7 @@
     </row>
     <row r="6" spans="1:4" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D6" s="12" t="s">
-        <v>2764</v>
+        <v>2767</v>
       </c>
     </row>
   </sheetData>
@@ -64983,180 +65428,180 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>2884</v>
+        <v>2897</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>2885</v>
+        <v>2898</v>
       </c>
       <c r="C1" s="13" t="s">
-        <v>2886</v>
+        <v>2899</v>
       </c>
       <c r="D1" s="13" t="s">
-        <v>2887</v>
+        <v>2900</v>
       </c>
       <c r="E1" s="13" t="s">
-        <v>2888</v>
+        <v>2901</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C2" s="14" t="s">
         <v>24</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>2891</v>
+        <v>2904</v>
       </c>
       <c r="E2" s="18" t="s">
-        <v>2916</v>
+        <v>2928</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>67</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>2893</v>
+        <v>2906</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>2917</v>
+        <v>2929</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>71</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>2896</v>
+        <v>2909</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>2918</v>
+        <v>2930</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>2688</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>2919</v>
+        <v>2931</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>2920</v>
+        <v>2932</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>2890</v>
+        <v>2903</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>2725</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>2898</v>
+        <v>2911</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>2899</v>
+        <v>2912</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>2900</v>
+        <v>2913</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>2709</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>2921</v>
+        <v>2933</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>2922</v>
+        <v>2934</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>2900</v>
+        <v>2913</v>
       </c>
       <c r="C8" s="12" t="s">
         <v>37</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>2903</v>
+        <v>2916</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>2904</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>2900</v>
+        <v>2913</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>2693</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>2923</v>
+        <v>2935</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>2924</v>
+        <v>2936</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>2925</v>
+        <v>2937</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>2882</v>
+        <v>2895</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>2926</v>
+        <v>2938</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>2927</v>
+        <v>2939</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>2925</v>
+        <v>2937</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>198</v>
@@ -65165,15 +65610,15 @@
         <v>23</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>2908</v>
+        <v>2921</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>2915</v>
+        <v>2927</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>2925</v>
+        <v>2937</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>363</v>
@@ -65182,7 +65627,7 @@
         <v>23</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>2909</v>
+        <v>2922</v>
       </c>
     </row>
   </sheetData>
@@ -65201,7 +65646,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="285" t="s">
-        <v>2928</v>
+        <v>2940</v>
       </c>
       <c r="B1" s="285"/>
       <c r="C1" s="285"/>
@@ -65211,7 +65656,7 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="286" t="s">
-        <v>2929</v>
+        <v>2941</v>
       </c>
       <c r="B2" s="286"/>
       <c r="C2" s="286"/>
@@ -65224,33 +65669,33 @@
         <v>19</v>
       </c>
       <c r="B4" s="102" t="s">
-        <v>2818</v>
+        <v>2830</v>
       </c>
       <c r="C4" s="102" t="s">
-        <v>2819</v>
+        <v>2831</v>
       </c>
       <c r="D4" s="102" t="s">
-        <v>2930</v>
+        <v>2942</v>
       </c>
       <c r="E4" s="102" t="s">
-        <v>2820</v>
+        <v>2832</v>
       </c>
       <c r="F4" s="102" t="s">
-        <v>2931</v>
+        <v>2943</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="str" cm="1">
-        <f t="array" ref="A5:A30">IFERROR(_xlfn._xlws.SORT(_xlfn.UNIQUE(_xlfn._xlws.FILTER(_xlfn.VSTACK('GECC 2026'!F2:F200,'GECC 2026'!AD3:AD32),_xlfn.VSTACK('GECC 2026'!F2:F200,'GECC 2026'!AD3:AD32)&lt;&gt;""))),"")</f>
-        <v>Adriana Cuoco Portugal</v>
+        <f t="array" ref="A5:A34">IFERROR(_xlfn._xlws.SORT(_xlfn.UNIQUE(_xlfn._xlws.FILTER(_xlfn.VSTACK('GECC 2026'!F2:F200,'GECC 2026'!AD3:AD32),_xlfn.VSTACK('GECC 2026'!F2:F200,'GECC 2026'!AD3:AD32)&lt;&gt;""))),"")</f>
+        <v>0</v>
       </c>
       <c r="B5" s="103">
         <f>IF($A5="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A5))</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C5" s="103">
         <f>IF($A5="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A5))</f>
-        <v>3.84</v>
+        <v>2.4</v>
       </c>
       <c r="D5" s="256">
         <f>IF($A5="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A5))</f>
@@ -65258,11 +65703,11 @@
       </c>
       <c r="E5" s="241">
         <f>IF($A5="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A5)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A5))</f>
-        <v>19.84</v>
+        <v>10.4</v>
       </c>
       <c r="F5" s="101">
         <f>IF($A5="","",COUNTIFS('GECC 2026'!F$2:F$200,$A5))</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G5" s="101">
         <f>IF($A5="","",COUNTIFS('GECC 2026'!G$2:G$200,$A5))</f>
@@ -65271,15 +65716,15 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="str">
-        <v>Adriana Magalhães</v>
+        <v>Adriana Cuoco Portugal</v>
       </c>
       <c r="B6" s="103">
         <f>IF($A6="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A6))</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C6" s="103">
         <f>IF($A6="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A6))</f>
-        <v>3.5999999999999996</v>
+        <v>3.84</v>
       </c>
       <c r="D6" s="256">
         <f>IF($A6="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A6))</f>
@@ -65287,24 +65732,24 @@
       </c>
       <c r="E6" s="241">
         <f>IF($A6="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A6)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A6))</f>
-        <v>27.6</v>
+        <v>19.84</v>
       </c>
       <c r="F6" s="101">
         <f>IF($A6="","",COUNTIFS('GECC 2026'!F$2:F$200,$A6))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="str">
-        <v>Arthur Wú</v>
+        <v>Adriana Magalhães</v>
       </c>
       <c r="B7" s="103">
         <f>IF($A7="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A7))</f>
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="C7" s="103">
         <f>IF($A7="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A7))</f>
-        <v>10.199999999999999</v>
+        <v>3.5999999999999996</v>
       </c>
       <c r="D7" s="256">
         <f>IF($A7="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A7))</f>
@@ -65312,74 +65757,74 @@
       </c>
       <c r="E7" s="241">
         <f>IF($A7="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A7)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A7))</f>
-        <v>43.2</v>
+        <v>27.6</v>
       </c>
       <c r="F7" s="101">
         <f>IF($A7="","",COUNTIFS('GECC 2026'!F$2:F$200,$A7))</f>
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="str">
-        <v>Cássio Murilo Alves Costa Filho</v>
+        <v>Arthur Wú</v>
       </c>
       <c r="B8" s="103">
         <f>IF($A8="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A8))</f>
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="C8" s="103">
         <f>IF($A8="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A8))</f>
-        <v>4.8</v>
+        <v>10.199999999999999</v>
       </c>
       <c r="D8" s="256">
         <f>IF($A8="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A8))</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E8" s="241">
         <f>IF($A8="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A8)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A8))</f>
-        <v>36.799999999999997</v>
+        <v>43.2</v>
       </c>
       <c r="F8" s="101">
         <f>IF($A8="","",COUNTIFS('GECC 2026'!F$2:F$200,$A8))</f>
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="str">
-        <v>Cinthia Thais de Carvalho Luz Thomazi</v>
+        <v>Cássio Murilo Alves Costa Filho</v>
       </c>
       <c r="B9" s="103">
         <f>IF($A9="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A9))</f>
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="C9" s="103">
         <f>IF($A9="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A9))</f>
-        <v>6.24</v>
+        <v>4.8</v>
       </c>
       <c r="D9" s="256">
         <f>IF($A9="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A9))</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E9" s="241">
         <f>IF($A9="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A9)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A9))</f>
-        <v>42.24</v>
+        <v>36.799999999999997</v>
       </c>
       <c r="F9" s="101">
         <f>IF($A9="","",COUNTIFS('GECC 2026'!F$2:F$200,$A9))</f>
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="str">
-        <v>Denise Duarte Guirra Kuhlmann</v>
+        <v>Cinthia Thais de Carvalho Luz Thomazi</v>
       </c>
       <c r="B10" s="103">
         <f>IF($A10="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A10))</f>
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="C10" s="103">
         <f>IF($A10="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A10))</f>
-        <v>2.6399999999999997</v>
+        <v>6.24</v>
       </c>
       <c r="D10" s="256">
         <f>IF($A10="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A10))</f>
@@ -65387,24 +65832,24 @@
       </c>
       <c r="E10" s="241">
         <f>IF($A10="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A10)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A10))</f>
-        <v>14.64</v>
+        <v>42.24</v>
       </c>
       <c r="F10" s="101">
         <f>IF($A10="","",COUNTIFS('GECC 2026'!F$2:F$200,$A10))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="str">
-        <v>Diversos</v>
+        <v>Davi Assunção Salvador Nery de Castro</v>
       </c>
       <c r="B11" s="103">
         <f>IF($A11="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A11))</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C11" s="103">
         <f>IF($A11="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A11))</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D11" s="256">
         <f>IF($A11="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A11))</f>
@@ -65412,7 +65857,7 @@
       </c>
       <c r="E11" s="241">
         <f>IF($A11="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A11)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A11))</f>
-        <v>0</v>
+        <v>13.2</v>
       </c>
       <c r="F11" s="101">
         <f>IF($A11="","",COUNTIFS('GECC 2026'!F$2:F$200,$A11))</f>
@@ -65421,15 +65866,15 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="str">
-        <v>Fernanda Viana de Souza</v>
+        <v>David da Silva de Araújo</v>
       </c>
       <c r="B12" s="103">
         <f>IF($A12="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A12))</f>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C12" s="103">
         <f>IF($A12="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A12))</f>
-        <v>3.09</v>
+        <v>1.2</v>
       </c>
       <c r="D12" s="256">
         <f>IF($A12="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A12))</f>
@@ -65437,24 +65882,24 @@
       </c>
       <c r="E12" s="241">
         <f>IF($A12="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A12)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A12))</f>
-        <v>18.09</v>
+        <v>13.2</v>
       </c>
       <c r="F12" s="101">
         <f>IF($A12="","",COUNTIFS('GECC 2026'!F$2:F$200,$A12))</f>
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="str">
-        <v>Flávio José Fonseca de Souza</v>
+        <v>Denise Duarte Guirra Kuhlmann</v>
       </c>
       <c r="B13" s="103">
         <f>IF($A13="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A13))</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C13" s="103">
         <f>IF($A13="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A13))</f>
-        <v>2.4</v>
+        <v>2.6399999999999997</v>
       </c>
       <c r="D13" s="256">
         <f>IF($A13="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A13))</f>
@@ -65462,24 +65907,24 @@
       </c>
       <c r="E13" s="241">
         <f>IF($A13="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A13)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A13))</f>
-        <v>10.4</v>
+        <v>14.64</v>
       </c>
       <c r="F13" s="101">
         <f>IF($A13="","",COUNTIFS('GECC 2026'!F$2:F$200,$A13))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
-        <v>Gabriel Heller</v>
+        <v>Diversos</v>
       </c>
       <c r="B14" s="103">
         <f>IF($A14="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A14))</f>
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="C14" s="103">
         <f>IF($A14="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A14))</f>
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="D14" s="256">
         <f>IF($A14="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A14))</f>
@@ -65487,7 +65932,7 @@
       </c>
       <c r="E14" s="241">
         <f>IF($A14="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A14)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A14))</f>
-        <v>37.200000000000003</v>
+        <v>0</v>
       </c>
       <c r="F14" s="101">
         <f>IF($A14="","",COUNTIFS('GECC 2026'!F$2:F$200,$A14))</f>
@@ -65496,15 +65941,15 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
-        <v>Gustavo Takahashi</v>
+        <v>Fernanda Viana de Souza</v>
       </c>
       <c r="B15" s="103">
         <f>IF($A15="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A15))</f>
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="C15" s="103">
         <f>IF($A15="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A15))</f>
-        <v>0</v>
+        <v>3.09</v>
       </c>
       <c r="D15" s="256">
         <f>IF($A15="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A15))</f>
@@ -65512,7 +65957,7 @@
       </c>
       <c r="E15" s="241">
         <f>IF($A15="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A15)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A15))</f>
-        <v>25</v>
+        <v>18.09</v>
       </c>
       <c r="F15" s="101">
         <f>IF($A15="","",COUNTIFS('GECC 2026'!F$2:F$200,$A15))</f>
@@ -65521,15 +65966,15 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
-        <v>Indio Artiaga do Brasil Rabelo</v>
+        <v>Flávio José Fonseca de Souza</v>
       </c>
       <c r="B16" s="103">
         <f>IF($A16="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A16))</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C16" s="103">
         <f>IF($A16="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A16))</f>
-        <v>3.6</v>
+        <v>2.4</v>
       </c>
       <c r="D16" s="256">
         <f>IF($A16="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A16))</f>
@@ -65537,7 +65982,7 @@
       </c>
       <c r="E16" s="241">
         <f>IF($A16="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A16)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A16))</f>
-        <v>15.6</v>
+        <v>10.4</v>
       </c>
       <c r="F16" s="101">
         <f>IF($A16="","",COUNTIFS('GECC 2026'!F$2:F$200,$A16))</f>
@@ -65546,15 +65991,15 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="str">
-        <v>Leonardo de Melo</v>
+        <v>Gabriel Heller</v>
       </c>
       <c r="B17" s="103">
         <f>IF($A17="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A17))</f>
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="C17" s="103">
         <f>IF($A17="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A17))</f>
-        <v>0</v>
+        <v>1.2</v>
       </c>
       <c r="D17" s="256">
         <f>IF($A17="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A17))</f>
@@ -65562,24 +66007,24 @@
       </c>
       <c r="E17" s="241">
         <f>IF($A17="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A17)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A17))</f>
-        <v>0</v>
+        <v>37.200000000000003</v>
       </c>
       <c r="F17" s="101">
         <f>IF($A17="","",COUNTIFS('GECC 2026'!F$2:F$200,$A17))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
-        <v>Leonardo José Alves Leal Neri</v>
+        <v>Gustavo Takahashi</v>
       </c>
       <c r="B18" s="103">
         <f>IF($A18="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A18))</f>
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="C18" s="103">
         <f>IF($A18="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A18))</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="D18" s="256">
         <f>IF($A18="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A18))</f>
@@ -65587,24 +66032,24 @@
       </c>
       <c r="E18" s="241">
         <f>IF($A18="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A18)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A18))</f>
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="F18" s="101">
         <f>IF($A18="","",COUNTIFS('GECC 2026'!F$2:F$200,$A18))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="str">
-        <v>Luciana Alvim</v>
+        <v>Hamilton de Jesus Lopes Neto</v>
       </c>
       <c r="B19" s="103">
         <f>IF($A19="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A19))</f>
-        <v>60</v>
+        <v>12</v>
       </c>
       <c r="C19" s="103">
         <f>IF($A19="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A19))</f>
-        <v>94</v>
+        <v>1.2</v>
       </c>
       <c r="D19" s="256">
         <f>IF($A19="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A19))</f>
@@ -65612,41 +66057,41 @@
       </c>
       <c r="E19" s="241">
         <f>IF($A19="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A19)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A19))</f>
-        <v>154</v>
+        <v>13.2</v>
       </c>
       <c r="F19" s="101">
         <f>IF($A19="","",COUNTIFS('GECC 2026'!F$2:F$200,$A19))</f>
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="str">
-        <v>Marcelo Bálbio Moraes</v>
+        <v>Indio Artiaga do Brasil Rabelo</v>
       </c>
       <c r="B20" s="103">
         <f>IF($A20="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A20))</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C20" s="103">
         <f>IF($A20="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A20))</f>
-        <v>0</v>
+        <v>3.6</v>
       </c>
       <c r="D20" s="256">
         <f>IF($A20="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A20))</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E20" s="241">
         <f>IF($A20="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A20)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A20))</f>
-        <v>16</v>
+        <v>15.6</v>
       </c>
       <c r="F20" s="101">
         <f>IF($A20="","",COUNTIFS('GECC 2026'!F$2:F$200,$A20))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="str">
-        <v>Mauri Siqueira Montessi</v>
+        <v>Leonardo de Melo</v>
       </c>
       <c r="B21" s="103">
         <f>IF($A21="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A21))</f>
@@ -65658,53 +66103,53 @@
       </c>
       <c r="D21" s="256">
         <f>IF($A21="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A21))</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E21" s="241">
         <f>IF($A21="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A21)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A21))</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="F21" s="101">
         <f>IF($A21="","",COUNTIFS('GECC 2026'!F$2:F$200,$A21))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="str">
-        <v>Michel Martins de Morais</v>
+        <v>Leonardo José Alves Leal Neri</v>
       </c>
       <c r="B22" s="103">
         <f>IF($A22="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A22))</f>
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C22" s="103">
         <f>IF($A22="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A22))</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D22" s="256">
         <f>IF($A22="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A22))</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E22" s="241">
         <f>IF($A22="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A22)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A22))</f>
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="F22" s="101">
         <f>IF($A22="","",COUNTIFS('GECC 2026'!F$2:F$200,$A22))</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="str">
-        <v>Paulo José Góes Daltro</v>
+        <v>Luciana Alvim</v>
       </c>
       <c r="B23" s="103">
         <f>IF($A23="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A23))</f>
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="C23" s="103">
         <f>IF($A23="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A23))</f>
-        <v>4.8</v>
+        <v>94</v>
       </c>
       <c r="D23" s="256">
         <f>IF($A23="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A23))</f>
@@ -65712,124 +66157,124 @@
       </c>
       <c r="E23" s="241">
         <f>IF($A23="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A23)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A23))</f>
-        <v>20.8</v>
+        <v>154</v>
       </c>
       <c r="F23" s="101">
         <f>IF($A23="","",COUNTIFS('GECC 2026'!F$2:F$200,$A23))</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="str">
-        <v>Priscila Nolasco</v>
+        <v>Marcelo Bálbio Moraes</v>
       </c>
       <c r="B24" s="103">
         <f>IF($A24="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A24))</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C24" s="103">
         <f>IF($A24="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A24))</f>
-        <v>2.6399999999999997</v>
+        <v>0</v>
       </c>
       <c r="D24" s="256">
         <f>IF($A24="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A24))</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E24" s="241">
         <f>IF($A24="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A24)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A24))</f>
-        <v>14.64</v>
+        <v>16</v>
       </c>
       <c r="F24" s="101">
         <f>IF($A24="","",COUNTIFS('GECC 2026'!F$2:F$200,$A24))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="str">
-        <v>Reinaldo Alencar</v>
+        <v>Mauri Siqueira Montessi</v>
       </c>
       <c r="B25" s="103">
         <f>IF($A25="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A25))</f>
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="C25" s="103">
         <f>IF($A25="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A25))</f>
-        <v>7.1999999999999993</v>
+        <v>0</v>
       </c>
       <c r="D25" s="256">
         <f>IF($A25="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A25))</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E25" s="241">
         <f>IF($A25="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A25)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A25))</f>
-        <v>55.2</v>
+        <v>16</v>
       </c>
       <c r="F25" s="101">
         <f>IF($A25="","",COUNTIFS('GECC 2026'!F$2:F$200,$A25))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="str">
-        <v>Rogério Ribeiro</v>
+        <v>Michel Martins de Morais</v>
       </c>
       <c r="B26" s="103">
         <f>IF($A26="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A26))</f>
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="C26" s="103">
         <f>IF($A26="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A26))</f>
-        <v>7.1999999999999993</v>
+        <v>0</v>
       </c>
       <c r="D26" s="256">
         <f>IF($A26="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A26))</f>
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E26" s="241">
         <f>IF($A26="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A26)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A26))</f>
-        <v>55.2</v>
+        <v>16</v>
       </c>
       <c r="F26" s="101">
         <f>IF($A26="","",COUNTIFS('GECC 2026'!F$2:F$200,$A26))</f>
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="str">
-        <v>Rômulo Miranda Alvim</v>
+        <v>Paulo José Góes Daltro</v>
       </c>
       <c r="B27" s="103">
         <f>IF($A27="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A27))</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C27" s="103">
         <f>IF($A27="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A27))</f>
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="D27" s="256">
         <f>IF($A27="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A27))</f>
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E27" s="241">
         <f>IF($A27="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A27)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A27))</f>
-        <v>43.6</v>
+        <v>20.8</v>
       </c>
       <c r="F27" s="101">
         <f>IF($A27="","",COUNTIFS('GECC 2026'!F$2:F$200,$A27))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="str">
-        <v>Servidores, colaboradores e estagiários do TCDF</v>
+        <v>Priscila Nolasco</v>
       </c>
       <c r="B28" s="103">
         <f>IF($A28="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A28))</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C28" s="103">
         <f>IF($A28="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A28))</f>
-        <v>0</v>
+        <v>2.6399999999999997</v>
       </c>
       <c r="D28" s="256">
         <f>IF($A28="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A28))</f>
@@ -65837,24 +66282,24 @@
       </c>
       <c r="E28" s="241">
         <f>IF($A28="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A28)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A28))</f>
-        <v>0</v>
+        <v>14.64</v>
       </c>
       <c r="F28" s="101">
         <f>IF($A28="","",COUNTIFS('GECC 2026'!F$2:F$200,$A28))</f>
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="str">
-        <v>Tarsila Firmino Ely</v>
+        <v>Reinaldo Alencar</v>
       </c>
       <c r="B29" s="103">
         <f>IF($A29="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A29))</f>
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C29" s="103">
         <f>IF($A29="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A29))</f>
-        <v>96.4</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="D29" s="256">
         <f>IF($A29="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A29))</f>
@@ -65862,24 +66307,24 @@
       </c>
       <c r="E29" s="241">
         <f>IF($A29="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A29)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A29))</f>
-        <v>152.4</v>
+        <v>55.2</v>
       </c>
       <c r="F29" s="101">
         <f>IF($A29="","",COUNTIFS('GECC 2026'!F$2:F$200,$A29))</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="str">
-        <v>Túllio Herbeth Teixeira Moraes</v>
+        <v>Rogério Ribeiro</v>
       </c>
       <c r="B30" s="103">
         <f>IF($A30="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A30))</f>
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="C30" s="103">
         <f>IF($A30="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A30))</f>
-        <v>0.44999999999999996</v>
+        <v>7.1999999999999993</v>
       </c>
       <c r="D30" s="256">
         <f>IF($A30="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A30))</f>
@@ -65887,102 +66332,114 @@
       </c>
       <c r="E30" s="241">
         <f>IF($A30="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A30)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A30))</f>
-        <v>3.45</v>
+        <v>55.2</v>
       </c>
       <c r="F30" s="101">
         <f>IF($A30="","",COUNTIFS('GECC 2026'!F$2:F$200,$A30))</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
+        <v>Rômulo Miranda Alvim</v>
+      </c>
+      <c r="B31" s="103">
+        <f>IF($A31="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A31))</f>
+        <v>24</v>
+      </c>
+      <c r="C31" s="103">
+        <f>IF($A31="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A31))</f>
+        <v>3.6</v>
+      </c>
+      <c r="D31" s="256">
+        <f>IF($A31="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A31))</f>
+        <v>16</v>
+      </c>
+      <c r="E31" s="241">
+        <f>IF($A31="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A31)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A31))</f>
+        <v>43.6</v>
+      </c>
+      <c r="F31" s="101">
+        <f>IF($A31="","",COUNTIFS('GECC 2026'!F$2:F$200,$A31))</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="str">
+        <v>Servidores, colaboradores e estagiários do TCDF</v>
+      </c>
+      <c r="B32" s="103">
+        <f>IF($A32="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A32))</f>
+        <v>0</v>
+      </c>
+      <c r="C32" s="103">
+        <f>IF($A32="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A32))</f>
+        <v>0</v>
+      </c>
+      <c r="D32" s="256">
+        <f>IF($A32="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A32))</f>
+        <v>0</v>
+      </c>
+      <c r="E32" s="241">
+        <f>IF($A32="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A32)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A32))</f>
+        <v>0</v>
+      </c>
+      <c r="F32" s="101">
+        <f>IF($A32="","",COUNTIFS('GECC 2026'!F$2:F$200,$A32))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B31" s="103" t="str">
-        <f>IF($A31="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A31))</f>
-        <v/>
-      </c>
-      <c r="C31" s="103" t="str">
-        <f>IF($A31="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A31))</f>
-        <v/>
-      </c>
-      <c r="D31" s="256" t="str">
-        <f>IF($A31="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A31))</f>
-        <v/>
-      </c>
-      <c r="E31" s="241" t="str">
-        <f>IF($A31="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A31)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A31))</f>
-        <v/>
-      </c>
-      <c r="F31" s="101" t="str">
-        <f>IF($A31="","",COUNTIFS('GECC 2026'!F$2:F$200,$A31))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B32" s="103" t="str">
-        <f>IF($A32="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A32))</f>
-        <v/>
-      </c>
-      <c r="C32" s="103" t="str">
-        <f>IF($A32="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A32))</f>
-        <v/>
-      </c>
-      <c r="D32" s="256" t="str">
-        <f>IF($A32="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A32))</f>
-        <v/>
-      </c>
-      <c r="E32" s="241" t="str">
-        <f>IF($A32="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A32)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A32))</f>
-        <v/>
-      </c>
-      <c r="F32" s="101" t="str">
-        <f>IF($A32="","",COUNTIFS('GECC 2026'!F$2:F$200,$A32))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B33" s="103" t="str">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="str">
+        <v>Tarsila Firmino Ely</v>
+      </c>
+      <c r="B33" s="103">
         <f>IF($A33="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A33))</f>
-        <v/>
-      </c>
-      <c r="C33" s="103" t="str">
+        <v>56</v>
+      </c>
+      <c r="C33" s="103">
         <f>IF($A33="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A33))</f>
-        <v/>
-      </c>
-      <c r="D33" s="256" t="str">
+        <v>96.4</v>
+      </c>
+      <c r="D33" s="256">
         <f>IF($A33="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A33))</f>
-        <v/>
-      </c>
-      <c r="E33" s="241" t="str">
+        <v>0</v>
+      </c>
+      <c r="E33" s="241">
         <f>IF($A33="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A33)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A33))</f>
-        <v/>
-      </c>
-      <c r="F33" s="101" t="str">
+        <v>152.4</v>
+      </c>
+      <c r="F33" s="101">
         <f>IF($A33="","",COUNTIFS('GECC 2026'!F$2:F$200,$A33))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B34" s="103" t="str">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="str">
+        <v>Túllio Herbeth Teixeira Moraes</v>
+      </c>
+      <c r="B34" s="103">
         <f>IF($A34="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A34))</f>
-        <v/>
-      </c>
-      <c r="C34" s="103" t="str">
+        <v>3</v>
+      </c>
+      <c r="C34" s="103">
         <f>IF($A34="","",SUMIFS('GECC 2026'!I$2:I$200,'GECC 2026'!F$2:F$200,$A34))</f>
-        <v/>
-      </c>
-      <c r="D34" s="256" t="str">
+        <v>0.44999999999999996</v>
+      </c>
+      <c r="D34" s="256">
         <f>IF($A34="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A34))</f>
-        <v/>
-      </c>
-      <c r="E34" s="241" t="str">
+        <v>0</v>
+      </c>
+      <c r="E34" s="241">
         <f>IF($A34="","",SUMIFS('GECC 2026'!J$2:J$200,'GECC 2026'!F$2:F$200,$A34)+SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A34))</f>
-        <v/>
-      </c>
-      <c r="F34" s="101" t="str">
+        <v>3.45</v>
+      </c>
+      <c r="F34" s="101">
         <f>IF($A34="","",COUNTIFS('GECC 2026'!F$2:F$200,$A34))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B35" s="103" t="str">
         <f>IF($A35="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A35))</f>
         <v/>
@@ -66004,7 +66461,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B36" s="103" t="str">
         <f>IF($A36="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A36))</f>
         <v/>
@@ -66026,7 +66483,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B37" s="103" t="str">
         <f>IF($A37="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A37))</f>
         <v/>
@@ -66048,7 +66505,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B38" s="103" t="str">
         <f>IF($A38="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A38))</f>
         <v/>
@@ -66070,7 +66527,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B39" s="103" t="str">
         <f>IF($A39="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A39))</f>
         <v/>
@@ -66092,7 +66549,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B40" s="103" t="str">
         <f>IF($A40="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A40))</f>
         <v/>
@@ -66114,7 +66571,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B41" s="103" t="str">
         <f>IF($A41="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A41))</f>
         <v/>
@@ -66136,7 +66593,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B42" s="103" t="str">
         <f>IF($A42="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A42))</f>
         <v/>
@@ -66158,7 +66615,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B43" s="103" t="str">
         <f>IF($A43="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A43))</f>
         <v/>
@@ -66180,7 +66637,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B44" s="103" t="str">
         <f>IF($A44="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A44))</f>
         <v/>
@@ -66202,7 +66659,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B45" s="103" t="str">
         <f>IF($A45="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A45))</f>
         <v/>
@@ -66224,7 +66681,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B46" s="103" t="str">
         <f>IF($A46="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A46))</f>
         <v/>
@@ -66246,7 +66703,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B47" s="103" t="str">
         <f>IF($A47="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A47))</f>
         <v/>
@@ -66268,7 +66725,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B48" s="103" t="str">
         <f>IF($A48="","",SUMIFS('GECC 2026'!H$2:H$200,'GECC 2026'!F$2:F$200,$A48))</f>
         <v/>
@@ -67476,15 +67933,15 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" s="242" t="s">
-        <v>2876</v>
+        <v>2889</v>
       </c>
       <c r="B105" s="243">
         <f>SUM(B5:B100)</f>
-        <v>540</v>
+        <v>584</v>
       </c>
       <c r="C105" s="243">
         <f>SUM(C5:C100)</f>
-        <v>269.89999999999998</v>
+        <v>275.89999999999998</v>
       </c>
       <c r="D105" s="256">
         <f>IF($A105="","",SUMIFS('GECC 2026'!$AE$3:$AE$32,'GECC 2026'!$AD$3:$AD$32,$A105))</f>
@@ -67496,7 +67953,7 @@
       </c>
       <c r="F105" s="244">
         <f>SUM(F5:F100)</f>
-        <v>63</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -67527,7 +67984,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="35.1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="287" t="s">
-        <v>2932</v>
+        <v>2944</v>
       </c>
       <c r="B1" s="287"/>
       <c r="C1" s="287"/>
@@ -67539,20 +67996,20 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="130" t="s">
-        <v>2933</v>
+        <v>2945</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="288" t="s">
-        <v>2934</v>
+        <v>2946</v>
       </c>
       <c r="B4" s="289"/>
       <c r="D4" s="288" t="s">
-        <v>2935</v>
+        <v>2947</v>
       </c>
       <c r="E4" s="289"/>
       <c r="G4" s="288" t="s">
-        <v>2936</v>
+        <v>2948</v>
       </c>
       <c r="H4" s="289"/>
     </row>
@@ -67576,28 +68033,28 @@
     <row r="6" spans="1:8" ht="9.9499999999999993" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="7" spans="1:8" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="143" t="s">
-        <v>2937</v>
+        <v>2949</v>
       </c>
       <c r="B7" s="143" t="s">
-        <v>2938</v>
+        <v>2950</v>
       </c>
       <c r="C7" s="143" t="s">
         <v>1</v>
       </c>
       <c r="D7" s="143" t="s">
-        <v>2939</v>
+        <v>2951</v>
       </c>
       <c r="E7" s="143" t="s">
-        <v>2940</v>
+        <v>2952</v>
       </c>
       <c r="F7" s="143" t="s">
-        <v>2815</v>
+        <v>2827</v>
       </c>
       <c r="G7" s="143" t="s">
         <v>5</v>
       </c>
       <c r="H7" s="143" t="s">
-        <v>2941</v>
+        <v>2953</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>